<commit_message>
Add Working list sheet: address, guide, Hometrack, guide +20%
A four-column view for day-to-day use, as the first sheet. 'Guide price'
is the current guide on the same basis as the +20% column: October where
the lot was re-entered, September otherwise.

Status is not a column here, so it is carried by row shading - green for
in the October catalogue, red for sold prior - and the Checked list sheet
keeps the full detail.

Hometrack is written as a number where one exists (70 of 100) and left as
the source text otherwise, so the column sorts and filters.

Cached values re-patched across both sheets after the insert shifted the
sheet order, and re-verified (212 of 212, no mismatches).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Kgh51upqvBx4um6iPVc7Lf
</commit_message>
<xml_diff>
--- a/auction_xref/Auction lots - checked list.xlsx
+++ b/auction_xref/Auction lots - checked list.xlsx
@@ -7,11 +7,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Checked list" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Notes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Working list" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Checked list" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Notes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checked list'!$A$1:$O$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Working list'!$A$1:$D$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Checked list'!$A$1:$O$101</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -101,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -151,6 +153,26 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -516,6 +538,1807 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D101"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Guide price</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Hometrack valuation</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Guide +20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>10 Eider Close, Hayes, Middlesex, UB4 9TD</t>
+        </is>
+      </c>
+      <c r="B2" s="17" t="n">
+        <v>395000</v>
+      </c>
+      <c r="C2" s="17" t="n">
+        <v>458000</v>
+      </c>
+      <c r="D2" s="17">
+        <f>IFERROR(B2*1.2,"")</f>
+        <v>474000.0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>2102 Kew Eye Apartments, Ealing Road, Brentford, Middlesex, TW8 0GA</t>
+        </is>
+      </c>
+      <c r="B3" s="17" t="n">
+        <v>410000</v>
+      </c>
+      <c r="C3" s="17" t="n">
+        <v>499000</v>
+      </c>
+      <c r="D3" s="17">
+        <f>IFERROR(B3*1.2,"")</f>
+        <v>492000.0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Sandly Court, 39 Queens Road, Southport, Merseyside, PR9 9EX</t>
+        </is>
+      </c>
+      <c r="B4" s="17" t="n">
+        <v>320000</v>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D4" s="17">
+        <f>IFERROR(B4*1.2,"")</f>
+        <v>384000.0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Flat 3 Regatta Point, 1 Manilla Street, Canary Wharf, London, E14 8JZ</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="n">
+        <v>225000</v>
+      </c>
+      <c r="C5" s="17" t="n">
+        <v>370000</v>
+      </c>
+      <c r="D5" s="17">
+        <f>IFERROR(B5*1.2,"")</f>
+        <v>270000.0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Flat 11 Regatta Point, 1 Manilla Street, Canary Wharf, London, E14 8JZ</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="n">
+        <v>180000</v>
+      </c>
+      <c r="C6" s="17" t="n">
+        <v>303000</v>
+      </c>
+      <c r="D6" s="17">
+        <f>IFERROR(B6*1.2,"")</f>
+        <v>216000.0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>9 Victoria Road, Margate, Kent, CT9 1LN</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="n">
+        <v>90000</v>
+      </c>
+      <c r="C7" s="17" t="n">
+        <v>238000</v>
+      </c>
+      <c r="D7" s="17">
+        <f>IFERROR(B7*1.2,"")</f>
+        <v>108000.0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Flat 4, 280 Wimborne Road, Bournemouth, Dorset, BH3 7AT</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="n">
+        <v>45000</v>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D8" s="17">
+        <f>IFERROR(B8*1.2,"")</f>
+        <v>54000.0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Flat 105, 2 Moorfields, Liverpool, Merseyside, L2 2BS</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="n">
+        <v>20000</v>
+      </c>
+      <c r="C9" s="17" t="n">
+        <v>90000</v>
+      </c>
+      <c r="D9" s="17">
+        <f>IFERROR(B9*1.2,"")</f>
+        <v>24000.0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Apartment 006 New Bank House, 100 Queen Street, Sheffield, South Yorkshire, S1 2FA</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C10" s="17" t="n">
+        <v>58000</v>
+      </c>
+      <c r="D10" s="17">
+        <f>IFERROR(B10*1.2,"")</f>
+        <v>6000.0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Parking Space 31 Lollard Street, Lambeth, London, SE11 6PX</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C11" s="18" t="inlineStr">
+        <is>
+          <t>N/A - parking</t>
+        </is>
+      </c>
+      <c r="D11" s="17">
+        <f>IFERROR(B11*1.2,"")</f>
+        <v>6000.0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Parking Space at 99 Mile End Road, Tower Hamlets, London, E1 4UH</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>N/A - parking</t>
+        </is>
+      </c>
+      <c r="D12" s="17">
+        <f>IFERROR(B12*1.2,"")</f>
+        <v>6000.0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Garage at 1 The Chestnuts, Gwydor Road, Beckenham, Kent, BR3 4DU</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="n">
+        <v>8000</v>
+      </c>
+      <c r="C13" s="20" t="inlineStr">
+        <is>
+          <t>N/A - garage</t>
+        </is>
+      </c>
+      <c r="D13" s="19">
+        <f>IFERROR(B13*1.2,"")</f>
+        <v>9600.0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Land to the Rear of 103 Church Street, Broadstairs, Kent, CT10 2TX</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="n">
+        <v>10000</v>
+      </c>
+      <c r="C14" s="20" t="inlineStr">
+        <is>
+          <t>N/A - land</t>
+        </is>
+      </c>
+      <c r="D14" s="19">
+        <f>IFERROR(B14*1.2,"")</f>
+        <v>12000.0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>Land Adjacent to The Gables, Banters Lane, Great Leighs, Chelmsford, Essex, CM3 1NT</t>
+        </is>
+      </c>
+      <c r="B15" s="21" t="n">
+        <v>1150000</v>
+      </c>
+      <c r="C15" s="22" t="inlineStr">
+        <is>
+          <t>N/A - land</t>
+        </is>
+      </c>
+      <c r="D15" s="21">
+        <f>IFERROR(B15*1.2,"")</f>
+        <v>1380000.0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>52 Bushey Grove Road, Bushey, Hertfordshire, WD23 2JJ</t>
+        </is>
+      </c>
+      <c r="B16" s="21" t="n">
+        <v>875000</v>
+      </c>
+      <c r="C16" s="21" t="n">
+        <v>875000</v>
+      </c>
+      <c r="D16" s="21">
+        <f>IFERROR(B16*1.2,"")</f>
+        <v>1050000.0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>104 Graveney Road, Tooting, London, SW17 0EH</t>
+        </is>
+      </c>
+      <c r="B17" s="21" t="n">
+        <v>775000</v>
+      </c>
+      <c r="C17" s="21" t="n">
+        <v>900000</v>
+      </c>
+      <c r="D17" s="21">
+        <f>IFERROR(B17*1.2,"")</f>
+        <v>930000.0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>23 Selkirk Road, Tooting, London, SW17 0ER</t>
+        </is>
+      </c>
+      <c r="B18" s="21" t="n">
+        <v>775000</v>
+      </c>
+      <c r="C18" s="21" t="n">
+        <v>965000</v>
+      </c>
+      <c r="D18" s="21">
+        <f>IFERROR(B18*1.2,"")</f>
+        <v>930000.0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>63 Warner Road, Camberwell, London, SE5 9NE</t>
+        </is>
+      </c>
+      <c r="B19" s="21" t="n">
+        <v>725000</v>
+      </c>
+      <c r="C19" s="21" t="n">
+        <v>521000</v>
+      </c>
+      <c r="D19" s="21">
+        <f>IFERROR(B19*1.2,"")</f>
+        <v>870000.0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>9 Fallow Court Avenue, Finchley, London, N12 0EA</t>
+        </is>
+      </c>
+      <c r="B20" s="21" t="n">
+        <v>695000</v>
+      </c>
+      <c r="C20" s="21" t="n">
+        <v>731000</v>
+      </c>
+      <c r="D20" s="21">
+        <f>IFERROR(B20*1.2,"")</f>
+        <v>834000.0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>196A St. Ann's Hill, Wandsworth, London, SW18 2RT</t>
+        </is>
+      </c>
+      <c r="B21" s="21" t="n">
+        <v>600000</v>
+      </c>
+      <c r="C21" s="21" t="n">
+        <v>815000</v>
+      </c>
+      <c r="D21" s="21">
+        <f>IFERROR(B21*1.2,"")</f>
+        <v>720000.0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>68 St. Margarets Avenue, Whetstone, London, N20 9LJ</t>
+        </is>
+      </c>
+      <c r="B22" s="21" t="n">
+        <v>550000</v>
+      </c>
+      <c r="C22" s="21" t="n">
+        <v>775000</v>
+      </c>
+      <c r="D22" s="21">
+        <f>IFERROR(B22*1.2,"")</f>
+        <v>660000.0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>Holmshill House, Summerswood Lane, Borehamwood, Hertfordshire, WD6 5PG</t>
+        </is>
+      </c>
+      <c r="B23" s="21" t="n">
+        <v>525000</v>
+      </c>
+      <c r="C23" s="21" t="n">
+        <v>1250000</v>
+      </c>
+      <c r="D23" s="21">
+        <f>IFERROR(B23*1.2,"")</f>
+        <v>630000.0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>396 Forest Road, Walthamstow, London, E17 5JF</t>
+        </is>
+      </c>
+      <c r="B24" s="21" t="n">
+        <v>500000</v>
+      </c>
+      <c r="C24" s="21" t="n">
+        <v>468000</v>
+      </c>
+      <c r="D24" s="21">
+        <f>IFERROR(B24*1.2,"")</f>
+        <v>600000.0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>Flat 91 Celeste House, 1 Caversham Road, Colindale, London, NW4 4DT</t>
+        </is>
+      </c>
+      <c r="B25" s="21" t="n">
+        <v>500000</v>
+      </c>
+      <c r="C25" s="21" t="n">
+        <v>693000</v>
+      </c>
+      <c r="D25" s="21">
+        <f>IFERROR(B25*1.2,"")</f>
+        <v>600000.0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>78 Park Chase, Wembley, Middlesex, HA9 8EH</t>
+        </is>
+      </c>
+      <c r="B26" s="21" t="n">
+        <v>450000</v>
+      </c>
+      <c r="C26" s="21" t="n">
+        <v>463000</v>
+      </c>
+      <c r="D26" s="21">
+        <f>IFERROR(B26*1.2,"")</f>
+        <v>540000.0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>Archie Court, 43 Marina, St Leonards-on-Sea, East Sussex, TN38 0BE</t>
+        </is>
+      </c>
+      <c r="B27" s="21" t="n">
+        <v>450000</v>
+      </c>
+      <c r="C27" s="22" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D27" s="21">
+        <f>IFERROR(B27*1.2,"")</f>
+        <v>540000.0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>15 Palestine Grove, Colliers Wood, London, SW19 2QN</t>
+        </is>
+      </c>
+      <c r="B28" s="21" t="n">
+        <v>425000</v>
+      </c>
+      <c r="C28" s="21" t="n">
+        <v>581000</v>
+      </c>
+      <c r="D28" s="21">
+        <f>IFERROR(B28*1.2,"")</f>
+        <v>510000.0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>Flat 23, 2 Manilla Street, Canary Wharf, London, E14 8GB</t>
+        </is>
+      </c>
+      <c r="B29" s="21" t="n">
+        <v>350000</v>
+      </c>
+      <c r="C29" s="21" t="n">
+        <v>534000</v>
+      </c>
+      <c r="D29" s="21">
+        <f>IFERROR(B29*1.2,"")</f>
+        <v>420000.0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>2 Holliday Street, Berkhamsted, Hertfordshire, HP4 2EE</t>
+        </is>
+      </c>
+      <c r="B30" s="21" t="n">
+        <v>325000</v>
+      </c>
+      <c r="C30" s="21" t="n">
+        <v>491000</v>
+      </c>
+      <c r="D30" s="21">
+        <f>IFERROR(B30*1.2,"")</f>
+        <v>390000.0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>19 Jarvis Road, South Croydon, Surrey, CR2 6HW</t>
+        </is>
+      </c>
+      <c r="B31" s="21" t="n">
+        <v>300000</v>
+      </c>
+      <c r="C31" s="21" t="n">
+        <v>313000</v>
+      </c>
+      <c r="D31" s="21">
+        <f>IFERROR(B31*1.2,"")</f>
+        <v>360000.0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>73 Hampton Road, Teddington, Middlesex, TW11 0LA</t>
+        </is>
+      </c>
+      <c r="B32" s="21" t="n">
+        <v>300000</v>
+      </c>
+      <c r="C32" s="21" t="n">
+        <v>533000</v>
+      </c>
+      <c r="D32" s="21">
+        <f>IFERROR(B32*1.2,"")</f>
+        <v>360000.0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>21 Wyncham Avenue, Sidcup, Kent, DA15 8EU</t>
+        </is>
+      </c>
+      <c r="B33" s="21" t="n">
+        <v>295000</v>
+      </c>
+      <c r="C33" s="21" t="n">
+        <v>585000</v>
+      </c>
+      <c r="D33" s="21">
+        <f>IFERROR(B33*1.2,"")</f>
+        <v>354000.0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t>174B Bravington Road, Maida Vale, London, W9 3AP</t>
+        </is>
+      </c>
+      <c r="B34" s="21" t="n">
+        <v>295000</v>
+      </c>
+      <c r="C34" s="21" t="n">
+        <v>572000</v>
+      </c>
+      <c r="D34" s="21">
+        <f>IFERROR(B34*1.2,"")</f>
+        <v>354000.0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>17-19 Umberston Street, Tower Hamlets, London, E1 1PY</t>
+        </is>
+      </c>
+      <c r="B35" s="21" t="n">
+        <v>275000</v>
+      </c>
+      <c r="C35" s="22" t="inlineStr">
+        <is>
+          <t>N/A - commercial</t>
+        </is>
+      </c>
+      <c r="D35" s="21">
+        <f>IFERROR(B35*1.2,"")</f>
+        <v>330000.0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t>Land Adjacent to Esso, Hogg Lane, Grays, Essex, RM17 5JA</t>
+        </is>
+      </c>
+      <c r="B36" s="21" t="n">
+        <v>235000</v>
+      </c>
+      <c r="C36" s="22" t="inlineStr">
+        <is>
+          <t>N/A - land</t>
+        </is>
+      </c>
+      <c r="D36" s="21">
+        <f>IFERROR(B36*1.2,"")</f>
+        <v>282000.0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>98 Victoria Road North, Southsea, Hampshire, PO5 1QE</t>
+        </is>
+      </c>
+      <c r="B37" s="21" t="n">
+        <v>220000</v>
+      </c>
+      <c r="C37" s="21" t="n">
+        <v>269000</v>
+      </c>
+      <c r="D37" s="21">
+        <f>IFERROR(B37*1.2,"")</f>
+        <v>264000.0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="12" t="inlineStr">
+        <is>
+          <t>9 St Anns Court, 45 Sunningfields Road, Hendon, London, NW4 4QY</t>
+        </is>
+      </c>
+      <c r="B38" s="21" t="n">
+        <v>200000</v>
+      </c>
+      <c r="C38" s="21" t="n">
+        <v>250000</v>
+      </c>
+      <c r="D38" s="21">
+        <f>IFERROR(B38*1.2,"")</f>
+        <v>240000.0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t>Ground Floor and Basement Flat, 134 Gipsy Hill, Crystal Palace, London, SE19 1PW</t>
+        </is>
+      </c>
+      <c r="B39" s="21" t="n">
+        <v>200000</v>
+      </c>
+      <c r="C39" s="21" t="n">
+        <v>368000</v>
+      </c>
+      <c r="D39" s="21">
+        <f>IFERROR(B39*1.2,"")</f>
+        <v>240000.0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="12" t="inlineStr">
+        <is>
+          <t>Foelas Residential Home, Station Road, Llanrug, Caernarfon, Gwynedd, LL55 4BE</t>
+        </is>
+      </c>
+      <c r="B40" s="21" t="n">
+        <v>200000</v>
+      </c>
+      <c r="C40" s="22" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D40" s="21">
+        <f>IFERROR(B40*1.2,"")</f>
+        <v>240000.0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t>Unit 6-6B South Middleton Base, Greenwell Road, Aberdeen, AB12 3AX</t>
+        </is>
+      </c>
+      <c r="B41" s="21" t="n">
+        <v>200000</v>
+      </c>
+      <c r="C41" s="22" t="inlineStr">
+        <is>
+          <t>N/A - commercial</t>
+        </is>
+      </c>
+      <c r="D41" s="21">
+        <f>IFERROR(B41*1.2,"")</f>
+        <v>240000.0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="12" t="inlineStr">
+        <is>
+          <t>Flat 17 Forest Croft, Taymount Rise, Forest Hill, London, SE23 3UN</t>
+        </is>
+      </c>
+      <c r="B42" s="21" t="n">
+        <v>200000</v>
+      </c>
+      <c r="C42" s="21" t="n">
+        <v>256000</v>
+      </c>
+      <c r="D42" s="21">
+        <f>IFERROR(B42*1.2,"")</f>
+        <v>240000.0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="12" t="inlineStr">
+        <is>
+          <t>29 The Crescent, Eastbourne, East Sussex, BN20 8PX</t>
+        </is>
+      </c>
+      <c r="B43" s="21" t="n">
+        <v>200000</v>
+      </c>
+      <c r="C43" s="21" t="n">
+        <v>203000</v>
+      </c>
+      <c r="D43" s="21">
+        <f>IFERROR(B43*1.2,"")</f>
+        <v>240000.0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="12" t="inlineStr">
+        <is>
+          <t>21 Greenfield Road, Pulloxhill, Bedford, Bedfordshire, MK45 5EZ</t>
+        </is>
+      </c>
+      <c r="B44" s="21" t="n">
+        <v>200000</v>
+      </c>
+      <c r="C44" s="21" t="n">
+        <v>366000</v>
+      </c>
+      <c r="D44" s="21">
+        <f>IFERROR(B44*1.2,"")</f>
+        <v>240000.0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="12" t="inlineStr">
+        <is>
+          <t>21 Preston Lane, Lyneham, Chippenham, Wiltshire, SN15 4AR</t>
+        </is>
+      </c>
+      <c r="B45" s="21" t="n">
+        <v>200000</v>
+      </c>
+      <c r="C45" s="21" t="n">
+        <v>252000</v>
+      </c>
+      <c r="D45" s="21">
+        <f>IFERROR(B45*1.2,"")</f>
+        <v>240000.0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="12" t="inlineStr">
+        <is>
+          <t>103 Buckingham Road, Edgware, Middlesex, HA8 6NN</t>
+        </is>
+      </c>
+      <c r="B46" s="21" t="n">
+        <v>185000</v>
+      </c>
+      <c r="C46" s="21" t="n">
+        <v>190000</v>
+      </c>
+      <c r="D46" s="21">
+        <f>IFERROR(B46*1.2,"")</f>
+        <v>222000.0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="12" t="inlineStr">
+        <is>
+          <t>Flat 41 Latchingdon Court, 26 Forest Road, Walthamstow, London, E17 6JT</t>
+        </is>
+      </c>
+      <c r="B47" s="21" t="n">
+        <v>180000</v>
+      </c>
+      <c r="C47" s="21" t="n">
+        <v>333000</v>
+      </c>
+      <c r="D47" s="21">
+        <f>IFERROR(B47*1.2,"")</f>
+        <v>216000.0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="12" t="inlineStr">
+        <is>
+          <t>13 Hope Street, Crook, County Durham, DL15 9HS</t>
+        </is>
+      </c>
+      <c r="B48" s="21" t="n">
+        <v>175000</v>
+      </c>
+      <c r="C48" s="21" t="n">
+        <v>95000</v>
+      </c>
+      <c r="D48" s="21">
+        <f>IFERROR(B48*1.2,"")</f>
+        <v>210000.0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="12" t="inlineStr">
+        <is>
+          <t>Flat 43 Ferrydale Lodge, 48 Church Road, Hendon, London, NW4 4EW</t>
+        </is>
+      </c>
+      <c r="B49" s="21" t="n">
+        <v>170000</v>
+      </c>
+      <c r="C49" s="21" t="n">
+        <v>224000</v>
+      </c>
+      <c r="D49" s="21">
+        <f>IFERROR(B49*1.2,"")</f>
+        <v>204000.0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="12" t="inlineStr">
+        <is>
+          <t>325A London Road, Westcliff-on-Sea, Essex, SS0 7BX</t>
+        </is>
+      </c>
+      <c r="B50" s="21" t="n">
+        <v>160000</v>
+      </c>
+      <c r="C50" s="21" t="n">
+        <v>161000</v>
+      </c>
+      <c r="D50" s="21">
+        <f>IFERROR(B50*1.2,"")</f>
+        <v>192000.0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="12" t="inlineStr">
+        <is>
+          <t>71 Fakes Road, Hemsby, Great Yarmouth, Norfolk, NR29 4JL</t>
+        </is>
+      </c>
+      <c r="B51" s="21" t="n">
+        <v>160000</v>
+      </c>
+      <c r="C51" s="21" t="n">
+        <v>241000</v>
+      </c>
+      <c r="D51" s="21">
+        <f>IFERROR(B51*1.2,"")</f>
+        <v>192000.0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="12" t="inlineStr">
+        <is>
+          <t>Flat 4 Maple Court, 1 Lower Coombe Street, Croydon, Surrey, CR0 1AA</t>
+        </is>
+      </c>
+      <c r="B52" s="21" t="n">
+        <v>150000</v>
+      </c>
+      <c r="C52" s="21" t="n">
+        <v>248000</v>
+      </c>
+      <c r="D52" s="21">
+        <f>IFERROR(B52*1.2,"")</f>
+        <v>180000.0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="12" t="inlineStr">
+        <is>
+          <t>Flat 3, 9 Queensland Road, Highbury, London, N7 7FH</t>
+        </is>
+      </c>
+      <c r="B53" s="21" t="n">
+        <v>145000</v>
+      </c>
+      <c r="C53" s="21" t="n">
+        <v>297000</v>
+      </c>
+      <c r="D53" s="21">
+        <f>IFERROR(B53*1.2,"")</f>
+        <v>174000.0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="12" t="inlineStr">
+        <is>
+          <t>102-104 High Street, Redcar, Cleveland, TS10 3DL</t>
+        </is>
+      </c>
+      <c r="B54" s="21" t="n">
+        <v>140000</v>
+      </c>
+      <c r="C54" s="21" t="n">
+        <v>82000</v>
+      </c>
+      <c r="D54" s="21">
+        <f>IFERROR(B54*1.2,"")</f>
+        <v>168000.0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="12" t="inlineStr">
+        <is>
+          <t>1 Hunter House, Hunter Road, Guildford, Surrey, GU1 3LQ</t>
+        </is>
+      </c>
+      <c r="B55" s="21" t="n">
+        <v>140000</v>
+      </c>
+      <c r="C55" s="21" t="n">
+        <v>337000</v>
+      </c>
+      <c r="D55" s="21">
+        <f>IFERROR(B55*1.2,"")</f>
+        <v>168000.0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="12" t="inlineStr">
+        <is>
+          <t>Land on the North-East side of Looe Gardens, Ilford, Essex, IG6 2BJ</t>
+        </is>
+      </c>
+      <c r="B56" s="21" t="n">
+        <v>135000</v>
+      </c>
+      <c r="C56" s="22" t="inlineStr">
+        <is>
+          <t>N/A - land</t>
+        </is>
+      </c>
+      <c r="D56" s="21">
+        <f>IFERROR(B56*1.2,"")</f>
+        <v>162000.0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="12" t="inlineStr">
+        <is>
+          <t>30 Ancton Way, Bognor Regis, West Sussex, PO22 6JW</t>
+        </is>
+      </c>
+      <c r="B57" s="21" t="n">
+        <v>130000</v>
+      </c>
+      <c r="C57" s="21" t="n">
+        <v>186000</v>
+      </c>
+      <c r="D57" s="21">
+        <f>IFERROR(B57*1.2,"")</f>
+        <v>156000.0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="12" t="inlineStr">
+        <is>
+          <t>3 Dane Court, College House, St Albans, Hertfordshire, AL1 5NX</t>
+        </is>
+      </c>
+      <c r="B58" s="21" t="n">
+        <v>110000</v>
+      </c>
+      <c r="C58" s="21" t="n">
+        <v>174000</v>
+      </c>
+      <c r="D58" s="21">
+        <f>IFERROR(B58*1.2,"")</f>
+        <v>132000.0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="12" t="inlineStr">
+        <is>
+          <t>37 and 37A Trevenson Street, Camborne, Cornwall, TR14 8JD</t>
+        </is>
+      </c>
+      <c r="B59" s="21" t="n">
+        <v>100000</v>
+      </c>
+      <c r="C59" s="21" t="n">
+        <v>122000</v>
+      </c>
+      <c r="D59" s="21">
+        <f>IFERROR(B59*1.2,"")</f>
+        <v>120000.0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="12" t="inlineStr">
+        <is>
+          <t>The Bungalow, 1 Chapel Lane, Maidford, Towcester, Northamptonshire, NN12 8HU</t>
+        </is>
+      </c>
+      <c r="B60" s="21" t="n">
+        <v>100000</v>
+      </c>
+      <c r="C60" s="21" t="n">
+        <v>302000</v>
+      </c>
+      <c r="D60" s="21">
+        <f>IFERROR(B60*1.2,"")</f>
+        <v>120000.0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="12" t="inlineStr">
+        <is>
+          <t>27 West Road, Shoeburyness, Southend-on-Sea, Essex, SS3 9DR</t>
+        </is>
+      </c>
+      <c r="B61" s="21" t="n">
+        <v>100000</v>
+      </c>
+      <c r="C61" s="21" t="n">
+        <v>218000</v>
+      </c>
+      <c r="D61" s="21">
+        <f>IFERROR(B61*1.2,"")</f>
+        <v>120000.0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="12" t="inlineStr">
+        <is>
+          <t>Unit SU8, 5 Jubilee Way, Scunthorpe, North Lincolnshire, DN15 6RB</t>
+        </is>
+      </c>
+      <c r="B62" s="21" t="n">
+        <v>95000</v>
+      </c>
+      <c r="C62" s="22" t="inlineStr">
+        <is>
+          <t>N/A - retail</t>
+        </is>
+      </c>
+      <c r="D62" s="21">
+        <f>IFERROR(B62*1.2,"")</f>
+        <v>114000.0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="12" t="inlineStr">
+        <is>
+          <t>9 College Walk, Rotherham, South Yorkshire, S60 1QB</t>
+        </is>
+      </c>
+      <c r="B63" s="21" t="n">
+        <v>95000</v>
+      </c>
+      <c r="C63" s="22" t="inlineStr">
+        <is>
+          <t>N/A - retail</t>
+        </is>
+      </c>
+      <c r="D63" s="21">
+        <f>IFERROR(B63*1.2,"")</f>
+        <v>114000.0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="12" t="inlineStr">
+        <is>
+          <t>94A Middleton Grange Shopping Centre, Hartlepool, Cleveland, TS24 7RW</t>
+        </is>
+      </c>
+      <c r="B64" s="21" t="n">
+        <v>95000</v>
+      </c>
+      <c r="C64" s="22" t="inlineStr">
+        <is>
+          <t>N/A - retail</t>
+        </is>
+      </c>
+      <c r="D64" s="21">
+        <f>IFERROR(B64*1.2,"")</f>
+        <v>114000.0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="12" t="inlineStr">
+        <is>
+          <t>2 Garfield Street, Northampton, Northamptonshire, NN2 6NW</t>
+        </is>
+      </c>
+      <c r="B65" s="21" t="n">
+        <v>95000</v>
+      </c>
+      <c r="C65" s="21" t="n">
+        <v>250000</v>
+      </c>
+      <c r="D65" s="21">
+        <f>IFERROR(B65*1.2,"")</f>
+        <v>114000.0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="12" t="inlineStr">
+        <is>
+          <t>29A High Street, March, Cambridgeshire, PE15 0XA</t>
+        </is>
+      </c>
+      <c r="B66" s="21" t="n">
+        <v>95000</v>
+      </c>
+      <c r="C66" s="21" t="n">
+        <v>178000</v>
+      </c>
+      <c r="D66" s="21">
+        <f>IFERROR(B66*1.2,"")</f>
+        <v>114000.0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="12" t="inlineStr">
+        <is>
+          <t>Flat 2, 201 Waldegrave Road, Teddington, Richmond upon Thames, TW11 8LX</t>
+        </is>
+      </c>
+      <c r="B67" s="21" t="n">
+        <v>95000</v>
+      </c>
+      <c r="C67" s="21" t="n">
+        <v>362000</v>
+      </c>
+      <c r="D67" s="21">
+        <f>IFERROR(B67*1.2,"")</f>
+        <v>114000.0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="12" t="inlineStr">
+        <is>
+          <t>Apartment 43, 18 Church Street, Manchester, Lancashire, M4 1PN</t>
+        </is>
+      </c>
+      <c r="B68" s="21" t="n">
+        <v>90000</v>
+      </c>
+      <c r="C68" s="21" t="n">
+        <v>193000</v>
+      </c>
+      <c r="D68" s="21">
+        <f>IFERROR(B68*1.2,"")</f>
+        <v>108000.0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="12" t="inlineStr">
+        <is>
+          <t>29 Hervey Street, Lowestoft, Suffolk, NR32 2JG</t>
+        </is>
+      </c>
+      <c r="B69" s="21" t="n">
+        <v>75000</v>
+      </c>
+      <c r="C69" s="21" t="n">
+        <v>153000</v>
+      </c>
+      <c r="D69" s="21">
+        <f>IFERROR(B69*1.2,"")</f>
+        <v>90000.0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="12" t="inlineStr">
+        <is>
+          <t>36 Hobart Road, Weston-super-Mare, Avon, BS23 4QN</t>
+        </is>
+      </c>
+      <c r="B70" s="21" t="n">
+        <v>70000</v>
+      </c>
+      <c r="C70" s="21" t="n">
+        <v>129000</v>
+      </c>
+      <c r="D70" s="21">
+        <f>IFERROR(B70*1.2,"")</f>
+        <v>84000.0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="12" t="inlineStr">
+        <is>
+          <t>4 Nairn Court, Dock Road, Tilbury, Essex, RM18 7BY</t>
+        </is>
+      </c>
+      <c r="B71" s="21" t="n">
+        <v>60000</v>
+      </c>
+      <c r="C71" s="21" t="n">
+        <v>149000</v>
+      </c>
+      <c r="D71" s="21">
+        <f>IFERROR(B71*1.2,"")</f>
+        <v>72000.0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="12" t="inlineStr">
+        <is>
+          <t>9A Battle Hill, Hexham, Northumberland, NE46 1BA</t>
+        </is>
+      </c>
+      <c r="B72" s="21" t="n">
+        <v>50000</v>
+      </c>
+      <c r="C72" s="22" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D72" s="21">
+        <f>IFERROR(B72*1.2,"")</f>
+        <v>60000.0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="12" t="inlineStr">
+        <is>
+          <t>106 High Street, Redcar, Cleveland, TS10 3DL</t>
+        </is>
+      </c>
+      <c r="B73" s="21" t="n">
+        <v>50000</v>
+      </c>
+      <c r="C73" s="21" t="n">
+        <v>82000</v>
+      </c>
+      <c r="D73" s="21">
+        <f>IFERROR(B73*1.2,"")</f>
+        <v>60000.0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="12" t="inlineStr">
+        <is>
+          <t>The Vaults, Manor Road, Chatham, Kent, ME4 6HW</t>
+        </is>
+      </c>
+      <c r="B74" s="21" t="n">
+        <v>50000</v>
+      </c>
+      <c r="C74" s="21" t="n">
+        <v>379000</v>
+      </c>
+      <c r="D74" s="21">
+        <f>IFERROR(B74*1.2,"")</f>
+        <v>60000.0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="12" t="inlineStr">
+        <is>
+          <t>Land to the rear of 21 Greenfield Road, Pulloxhill, Bedford, Bedfordshire, MK45 5EZ</t>
+        </is>
+      </c>
+      <c r="B75" s="21" t="n">
+        <v>50000</v>
+      </c>
+      <c r="C75" s="22" t="inlineStr">
+        <is>
+          <t>N/A - land</t>
+        </is>
+      </c>
+      <c r="D75" s="21">
+        <f>IFERROR(B75*1.2,"")</f>
+        <v>60000.0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="12" t="inlineStr">
+        <is>
+          <t>Flat 3, 55 West Avenue, Filey, North Yorkshire, YO14 9AX</t>
+        </is>
+      </c>
+      <c r="B76" s="21" t="n">
+        <v>50000</v>
+      </c>
+      <c r="C76" s="21" t="n">
+        <v>130000</v>
+      </c>
+      <c r="D76" s="21">
+        <f>IFERROR(B76*1.2,"")</f>
+        <v>60000.0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="12" t="inlineStr">
+        <is>
+          <t>65 Reeves Road, Derby, Derbyshire, DE23 8JF</t>
+        </is>
+      </c>
+      <c r="B77" s="21" t="n">
+        <v>45000</v>
+      </c>
+      <c r="C77" s="21" t="n">
+        <v>87500</v>
+      </c>
+      <c r="D77" s="21">
+        <f>IFERROR(B77*1.2,"")</f>
+        <v>54000.0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="12" t="inlineStr">
+        <is>
+          <t>4 Milburn Street, Crook, County Durham, DL15 9DY</t>
+        </is>
+      </c>
+      <c r="B78" s="21" t="n">
+        <v>40000</v>
+      </c>
+      <c r="C78" s="21" t="n">
+        <v>92500</v>
+      </c>
+      <c r="D78" s="21">
+        <f>IFERROR(B78*1.2,"")</f>
+        <v>48000.0</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="12" t="inlineStr">
+        <is>
+          <t>Land to the rear of 141 Parsonage Road, Rainham, Essex, RM13 9LB</t>
+        </is>
+      </c>
+      <c r="B79" s="21" t="n">
+        <v>35000</v>
+      </c>
+      <c r="C79" s="22" t="inlineStr">
+        <is>
+          <t>N/A - land</t>
+        </is>
+      </c>
+      <c r="D79" s="21">
+        <f>IFERROR(B79*1.2,"")</f>
+        <v>42000.0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="12" t="inlineStr">
+        <is>
+          <t>49 Exmouth Road, Great Yarmouth, Norfolk, NR30 3DP</t>
+        </is>
+      </c>
+      <c r="B80" s="21" t="n">
+        <v>30000</v>
+      </c>
+      <c r="C80" s="21" t="n">
+        <v>81000</v>
+      </c>
+      <c r="D80" s="21">
+        <f>IFERROR(B80*1.2,"")</f>
+        <v>36000.0</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="12" t="inlineStr">
+        <is>
+          <t>34 Murton Lane, Easington Lane, Houghton Le Spring, Tyne and Wear, DH5 0NB</t>
+        </is>
+      </c>
+      <c r="B81" s="21" t="n">
+        <v>30000</v>
+      </c>
+      <c r="C81" s="21" t="n">
+        <v>40000</v>
+      </c>
+      <c r="D81" s="21">
+        <f>IFERROR(B81*1.2,"")</f>
+        <v>36000.0</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="12" t="inlineStr">
+        <is>
+          <t>Rear of 292 Weelsby Street, Grimsby, North East Lincolnshire, DN32 8AB</t>
+        </is>
+      </c>
+      <c r="B82" s="21" t="n">
+        <v>25000</v>
+      </c>
+      <c r="C82" s="22" t="inlineStr">
+        <is>
+          <t>N/A - workshop</t>
+        </is>
+      </c>
+      <c r="D82" s="21">
+        <f>IFERROR(B82*1.2,"")</f>
+        <v>30000.0</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="12" t="inlineStr">
+        <is>
+          <t>108 High Street, Redcar, Cleveland, TS10 3DL</t>
+        </is>
+      </c>
+      <c r="B83" s="21" t="n">
+        <v>25000</v>
+      </c>
+      <c r="C83" s="21" t="n">
+        <v>82000</v>
+      </c>
+      <c r="D83" s="21">
+        <f>IFERROR(B83*1.2,"")</f>
+        <v>30000.0</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="12" t="inlineStr">
+        <is>
+          <t>4 Highfield Road, Newbold, Derbyshire, S41 7EY</t>
+        </is>
+      </c>
+      <c r="B84" s="21" t="n">
+        <v>25000</v>
+      </c>
+      <c r="C84" s="21" t="n">
+        <v>310000</v>
+      </c>
+      <c r="D84" s="21">
+        <f>IFERROR(B84*1.2,"")</f>
+        <v>30000.0</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="12" t="inlineStr">
+        <is>
+          <t>Flat 110, 2 Moorfields, Liverpool, Merseyside, L2 2BS</t>
+        </is>
+      </c>
+      <c r="B85" s="21" t="n">
+        <v>20000</v>
+      </c>
+      <c r="C85" s="21" t="n">
+        <v>90000</v>
+      </c>
+      <c r="D85" s="21">
+        <f>IFERROR(B85*1.2,"")</f>
+        <v>24000.0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="12" t="inlineStr">
+        <is>
+          <t>Residential Flat, 9A Battle Hill, Hexham, Northumberland, NE46 1BA</t>
+        </is>
+      </c>
+      <c r="B86" s="21" t="n">
+        <v>20000</v>
+      </c>
+      <c r="C86" s="21" t="n">
+        <v>64500</v>
+      </c>
+      <c r="D86" s="21">
+        <f>IFERROR(B86*1.2,"")</f>
+        <v>24000.0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="12" t="inlineStr">
+        <is>
+          <t>Flat 29 The Old School Rooms, Great Moor Street, Bolton, Lancashire, BL1 1NR</t>
+        </is>
+      </c>
+      <c r="B87" s="21" t="n">
+        <v>20000</v>
+      </c>
+      <c r="C87" s="21" t="n">
+        <v>112000</v>
+      </c>
+      <c r="D87" s="21">
+        <f>IFERROR(B87*1.2,"")</f>
+        <v>24000.0</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="12" t="inlineStr">
+        <is>
+          <t>First &amp; Second Floor, 5 Cornmarket, Penrith, Cumbria, CA11 7DA</t>
+        </is>
+      </c>
+      <c r="B88" s="21" t="n">
+        <v>20000</v>
+      </c>
+      <c r="C88" s="21" t="n">
+        <v>136000</v>
+      </c>
+      <c r="D88" s="21">
+        <f>IFERROR(B88*1.2,"")</f>
+        <v>24000.0</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="12" t="inlineStr">
+        <is>
+          <t>2 Broad Street, St. Columb, Cornwall, TR9 6AS</t>
+        </is>
+      </c>
+      <c r="B89" s="21" t="n">
+        <v>15000</v>
+      </c>
+      <c r="C89" s="21" t="n">
+        <v>20500</v>
+      </c>
+      <c r="D89" s="21">
+        <f>IFERROR(B89*1.2,"")</f>
+        <v>18000.0</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="12" t="inlineStr">
+        <is>
+          <t>Land at Green Lane, Warlingham, Surrey, CR6 9EE</t>
+        </is>
+      </c>
+      <c r="B90" s="21" t="n">
+        <v>15000</v>
+      </c>
+      <c r="C90" s="22" t="inlineStr">
+        <is>
+          <t>N/A - land</t>
+        </is>
+      </c>
+      <c r="D90" s="21">
+        <f>IFERROR(B90*1.2,"")</f>
+        <v>18000.0</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="12" t="inlineStr">
+        <is>
+          <t>Unit 1 Masonic Hall, 64 Briggate, Brighouse, Calderdale, HD6 1EF</t>
+        </is>
+      </c>
+      <c r="B91" s="21" t="n">
+        <v>9000</v>
+      </c>
+      <c r="C91" s="22" t="inlineStr">
+        <is>
+          <t>N/A - commercial</t>
+        </is>
+      </c>
+      <c r="D91" s="21">
+        <f>IFERROR(B91*1.2,"")</f>
+        <v>10800.0</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="12" t="inlineStr">
+        <is>
+          <t>Unit 3, 6A Alma Street, Taunton, Somerset, TA1 3AH</t>
+        </is>
+      </c>
+      <c r="B92" s="21" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C92" s="22" t="inlineStr">
+        <is>
+          <t>N/A - commercial</t>
+        </is>
+      </c>
+      <c r="D92" s="21">
+        <f>IFERROR(B92*1.2,"")</f>
+        <v>6000.0</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="12" t="inlineStr">
+        <is>
+          <t>18 Farringford Court, 1 Avenue Road, Lymington, Hampshire, SO41 9PA</t>
+        </is>
+      </c>
+      <c r="B93" s="21" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C93" s="21" t="n">
+        <v>150000</v>
+      </c>
+      <c r="D93" s="21">
+        <f>IFERROR(B93*1.2,"")</f>
+        <v>6000.0</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="12" t="inlineStr">
+        <is>
+          <t>Flat A9-D Leighton Street, Leighton Street, Preston, Lancashire, PR1 8RH</t>
+        </is>
+      </c>
+      <c r="B94" s="21" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C94" s="22" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D94" s="21">
+        <f>IFERROR(B94*1.2,"")</f>
+        <v>6000.0</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="12" t="inlineStr">
+        <is>
+          <t>Plot 8 Boreham Place, New England, Halstead, Essex, CO9 4BD</t>
+        </is>
+      </c>
+      <c r="B95" s="21" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C95" s="22" t="inlineStr">
+        <is>
+          <t>N/A - plot</t>
+        </is>
+      </c>
+      <c r="D95" s="21">
+        <f>IFERROR(B95*1.2,"")</f>
+        <v>6000.0</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="12" t="inlineStr">
+        <is>
+          <t>Plot 4 Station Road, Shirehampton, Bristol, Avon, BS11 9XA</t>
+        </is>
+      </c>
+      <c r="B96" s="21" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C96" s="22" t="inlineStr">
+        <is>
+          <t>N/A - plot</t>
+        </is>
+      </c>
+      <c r="D96" s="21">
+        <f>IFERROR(B96*1.2,"")</f>
+        <v>6000.0</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="12" t="inlineStr">
+        <is>
+          <t>Garage and Land to the Rear of 16 Stanley Park Drive, Wembley, Middlesex, HA0 1SG</t>
+        </is>
+      </c>
+      <c r="B97" s="21" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C97" s="22" t="inlineStr">
+        <is>
+          <t>N/A - garage</t>
+        </is>
+      </c>
+      <c r="D97" s="21">
+        <f>IFERROR(B97*1.2,"")</f>
+        <v>6000.0</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="12" t="inlineStr">
+        <is>
+          <t>Garage at Seddon Court, Hepplewhite Close, Crawley, West Sussex, RH11 9LF</t>
+        </is>
+      </c>
+      <c r="B98" s="21" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C98" s="22" t="inlineStr">
+        <is>
+          <t>N/A - garage</t>
+        </is>
+      </c>
+      <c r="D98" s="21">
+        <f>IFERROR(B98*1.2,"")</f>
+        <v>6000.0</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="12" t="inlineStr">
+        <is>
+          <t>Plot 2 Abbey Street, Ickleton, Saffron Walden, Essex, CB10 1SS</t>
+        </is>
+      </c>
+      <c r="B99" s="21" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C99" s="22" t="inlineStr">
+        <is>
+          <t>N/A - plot</t>
+        </is>
+      </c>
+      <c r="D99" s="21">
+        <f>IFERROR(B99*1.2,"")</f>
+        <v>3600.0</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="12" t="inlineStr">
+        <is>
+          <t>Compound 1, Par Moor Road, Par, Cornwall, PL24 2SQ</t>
+        </is>
+      </c>
+      <c r="B100" s="21" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C100" s="22" t="inlineStr">
+        <is>
+          <t>N/A - compound</t>
+        </is>
+      </c>
+      <c r="D100" s="21">
+        <f>IFERROR(B100*1.2,"")</f>
+        <v>3600.0</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="12" t="inlineStr">
+        <is>
+          <t>Flat 201 Lemare Lodge, Fair Acres, Bromley, Kent, BR2 9BS</t>
+        </is>
+      </c>
+      <c r="B101" s="22" t="n"/>
+      <c r="C101" s="21" t="n">
+        <v>226000</v>
+      </c>
+      <c r="D101" s="21">
+        <f>IFERROR(B101*1.2,"")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D101"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:O101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -6397,13 +8220,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A55"/>
+  <dimension ref="A1:A63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -6754,6 +8577,55 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" s="23" t="inlineStr">
+        <is>
+          <t>Working list sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="24" t="inlineStr">
+        <is>
+          <t>Address / guide price / Hometrack valuation / guide +20%, for all 100 lots.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="24" t="inlineStr">
+        <is>
+          <t>'Guide price' is the CURRENT guide: the October guide where the lot was re-entered, the</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="24" t="inlineStr">
+        <is>
+          <t>September guide otherwise - the same basis as the +20% column. Range guides use the low end.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="24" t="inlineStr">
+        <is>
+          <t>Row shading carries the status, since it is not a column here: green = in the October</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="24" t="inlineStr">
+        <is>
+          <t>catalogue, red = sold prior, unshaded = not in the October catalogue. The 'Checked list'</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="24" t="inlineStr">
+        <is>
+          <t>sheet has the full detail including October lot numbers and how each match was verified.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Carry the accepted-offer column onto the Working list
Adds 'Offer likely accepted' from the source spreadsheet, plus offer as a
percentage of Hometrack so it sits alongside the guide+20% comparison.
26 lots carry a figure.

The 7 lots recorded as 'No offers' are labelled as such rather than left
blank: that is a result, not a missing value, and blanks would read as
never-pursued like the other 67.

Notes sheet records that these offers relate to the September sale, so on
a lot re-entered in October at a cut guide they may be stale - lot 166
carries a £35,000 offer against an October guide of £5,000-£15,000.

Cached values re-patched across both sheets again (307 cells, verified).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Kgh51upqvBx4um6iPVc7Lf
</commit_message>
<xml_diff>
--- a/auction_xref/Auction lots - checked list.xlsx
+++ b/auction_xref/Auction lots - checked list.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Notes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Working list'!$A$1:$E$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Working list'!$A$1:$G$101</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Checked list'!$A$1:$O$101</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -538,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E101"/>
+  <dimension ref="A1:G101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -546,6 +546,8 @@
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -574,6 +576,16 @@
           <t>Guide +20% as % of Hometrack</t>
         </is>
       </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Offer likely accepted (£)</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Offer as % of Hometrack</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -595,6 +607,11 @@
         <f>IFERROR(D2/C2,"")</f>
         <v>1.0349344978</v>
       </c>
+      <c r="F2" s="17" t="n"/>
+      <c r="G2" s="6">
+        <f>IFERROR(F2/C2,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -616,6 +633,11 @@
         <f>IFERROR(D3/C3,"")</f>
         <v>0.9859719439</v>
       </c>
+      <c r="F3" s="17" t="n"/>
+      <c r="G3" s="6">
+        <f>IFERROR(F3/C3,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -639,6 +661,11 @@
         <f>IFERROR(D4/C4,"")</f>
         <v/>
       </c>
+      <c r="F4" s="17" t="n"/>
+      <c r="G4" s="6">
+        <f>IFERROR(F4/C4,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -660,6 +687,11 @@
         <f>IFERROR(D5/C5,"")</f>
         <v>0.7297297297</v>
       </c>
+      <c r="F5" s="17" t="n"/>
+      <c r="G5" s="6">
+        <f>IFERROR(F5/C5,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -681,6 +713,11 @@
         <f>IFERROR(D6/C6,"")</f>
         <v>0.7128712871</v>
       </c>
+      <c r="F6" s="17" t="n"/>
+      <c r="G6" s="6">
+        <f>IFERROR(F6/C6,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -702,6 +739,15 @@
         <f>IFERROR(D7/C7,"")</f>
         <v>0.4537815126</v>
       </c>
+      <c r="F7" s="17" t="inlineStr">
+        <is>
+          <t>No offers</t>
+        </is>
+      </c>
+      <c r="G7" s="6">
+        <f>IFERROR(F7/C7,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -725,6 +771,11 @@
         <f>IFERROR(D8/C8,"")</f>
         <v/>
       </c>
+      <c r="F8" s="17" t="n"/>
+      <c r="G8" s="6">
+        <f>IFERROR(F8/C8,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -746,6 +797,13 @@
         <f>IFERROR(D9/C9,"")</f>
         <v>0.2666666667</v>
       </c>
+      <c r="F9" s="17" t="n">
+        <v>40000</v>
+      </c>
+      <c r="G9" s="6">
+        <f>IFERROR(F9/C9,"")</f>
+        <v>0.4444444444</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -767,6 +825,13 @@
         <f>IFERROR(D10/C10,"")</f>
         <v>0.1034482759</v>
       </c>
+      <c r="F10" s="17" t="n">
+        <v>35000</v>
+      </c>
+      <c r="G10" s="6">
+        <f>IFERROR(F10/C10,"")</f>
+        <v>0.6034482759</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -790,6 +855,11 @@
         <f>IFERROR(D11/C11,"")</f>
         <v/>
       </c>
+      <c r="F11" s="17" t="n"/>
+      <c r="G11" s="6">
+        <f>IFERROR(F11/C11,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -813,6 +883,11 @@
         <f>IFERROR(D12/C12,"")</f>
         <v/>
       </c>
+      <c r="F12" s="17" t="n"/>
+      <c r="G12" s="6">
+        <f>IFERROR(F12/C12,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
@@ -836,6 +911,11 @@
         <f>IFERROR(D13/C13,"")</f>
         <v/>
       </c>
+      <c r="F13" s="19" t="n"/>
+      <c r="G13" s="10">
+        <f>IFERROR(F13/C13,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
@@ -859,6 +939,11 @@
         <f>IFERROR(D14/C14,"")</f>
         <v/>
       </c>
+      <c r="F14" s="19" t="n"/>
+      <c r="G14" s="10">
+        <f>IFERROR(F14/C14,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
@@ -882,6 +967,11 @@
         <f>IFERROR(D15/C15,"")</f>
         <v/>
       </c>
+      <c r="F15" s="21" t="n"/>
+      <c r="G15" s="14">
+        <f>IFERROR(F15/C15,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
@@ -903,6 +993,11 @@
         <f>IFERROR(D16/C16,"")</f>
         <v>1.2</v>
       </c>
+      <c r="F16" s="21" t="n"/>
+      <c r="G16" s="14">
+        <f>IFERROR(F16/C16,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
@@ -924,6 +1019,11 @@
         <f>IFERROR(D17/C17,"")</f>
         <v>1.0333333333</v>
       </c>
+      <c r="F17" s="21" t="n"/>
+      <c r="G17" s="14">
+        <f>IFERROR(F17/C17,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
@@ -945,6 +1045,11 @@
         <f>IFERROR(D18/C18,"")</f>
         <v>0.9637305699</v>
       </c>
+      <c r="F18" s="21" t="n"/>
+      <c r="G18" s="14">
+        <f>IFERROR(F18/C18,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
@@ -966,6 +1071,11 @@
         <f>IFERROR(D19/C19,"")</f>
         <v>1.669865643</v>
       </c>
+      <c r="F19" s="21" t="n"/>
+      <c r="G19" s="14">
+        <f>IFERROR(F19/C19,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
@@ -987,6 +1097,11 @@
         <f>IFERROR(D20/C20,"")</f>
         <v>1.1409028728</v>
       </c>
+      <c r="F20" s="21" t="n"/>
+      <c r="G20" s="14">
+        <f>IFERROR(F20/C20,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
@@ -1008,6 +1123,11 @@
         <f>IFERROR(D21/C21,"")</f>
         <v>0.8834355828</v>
       </c>
+      <c r="F21" s="21" t="n"/>
+      <c r="G21" s="14">
+        <f>IFERROR(F21/C21,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
@@ -1029,6 +1149,11 @@
         <f>IFERROR(D22/C22,"")</f>
         <v>0.8516129032</v>
       </c>
+      <c r="F22" s="21" t="n"/>
+      <c r="G22" s="14">
+        <f>IFERROR(F22/C22,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
@@ -1050,6 +1175,13 @@
         <f>IFERROR(D23/C23,"")</f>
         <v>0.504</v>
       </c>
+      <c r="F23" s="21" t="n">
+        <v>625000</v>
+      </c>
+      <c r="G23" s="14">
+        <f>IFERROR(F23/C23,"")</f>
+        <v>0.5</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
@@ -1071,6 +1203,11 @@
         <f>IFERROR(D24/C24,"")</f>
         <v>1.2820512821</v>
       </c>
+      <c r="F24" s="21" t="n"/>
+      <c r="G24" s="14">
+        <f>IFERROR(F24/C24,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
@@ -1092,6 +1229,11 @@
         <f>IFERROR(D25/C25,"")</f>
         <v>0.8658008658</v>
       </c>
+      <c r="F25" s="21" t="n"/>
+      <c r="G25" s="14">
+        <f>IFERROR(F25/C25,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
@@ -1113,6 +1255,11 @@
         <f>IFERROR(D26/C26,"")</f>
         <v>1.1663066955</v>
       </c>
+      <c r="F26" s="21" t="n"/>
+      <c r="G26" s="14">
+        <f>IFERROR(F26/C26,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
@@ -1136,6 +1283,11 @@
         <f>IFERROR(D27/C27,"")</f>
         <v/>
       </c>
+      <c r="F27" s="21" t="n"/>
+      <c r="G27" s="14">
+        <f>IFERROR(F27/C27,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="12" t="inlineStr">
@@ -1157,6 +1309,11 @@
         <f>IFERROR(D28/C28,"")</f>
         <v>0.8777969019</v>
       </c>
+      <c r="F28" s="21" t="n"/>
+      <c r="G28" s="14">
+        <f>IFERROR(F28/C28,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
@@ -1178,6 +1335,11 @@
         <f>IFERROR(D29/C29,"")</f>
         <v>0.7865168539</v>
       </c>
+      <c r="F29" s="21" t="n"/>
+      <c r="G29" s="14">
+        <f>IFERROR(F29/C29,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="12" t="inlineStr">
@@ -1199,6 +1361,11 @@
         <f>IFERROR(D30/C30,"")</f>
         <v>0.7942973523</v>
       </c>
+      <c r="F30" s="21" t="n"/>
+      <c r="G30" s="14">
+        <f>IFERROR(F30/C30,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="12" t="inlineStr">
@@ -1220,6 +1387,11 @@
         <f>IFERROR(D31/C31,"")</f>
         <v>1.1501597444</v>
       </c>
+      <c r="F31" s="21" t="n"/>
+      <c r="G31" s="14">
+        <f>IFERROR(F31/C31,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="12" t="inlineStr">
@@ -1241,6 +1413,15 @@
         <f>IFERROR(D32/C32,"")</f>
         <v>0.6754221388</v>
       </c>
+      <c r="F32" s="21" t="inlineStr">
+        <is>
+          <t>No offers</t>
+        </is>
+      </c>
+      <c r="G32" s="14">
+        <f>IFERROR(F32/C32,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="12" t="inlineStr">
@@ -1262,6 +1443,13 @@
         <f>IFERROR(D33/C33,"")</f>
         <v>0.6051282051</v>
       </c>
+      <c r="F33" s="21" t="n">
+        <v>325000</v>
+      </c>
+      <c r="G33" s="14">
+        <f>IFERROR(F33/C33,"")</f>
+        <v>0.5555555556</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="12" t="inlineStr">
@@ -1283,6 +1471,15 @@
         <f>IFERROR(D34/C34,"")</f>
         <v>0.6188811189</v>
       </c>
+      <c r="F34" s="21" t="inlineStr">
+        <is>
+          <t>No offers</t>
+        </is>
+      </c>
+      <c r="G34" s="14">
+        <f>IFERROR(F34/C34,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="12" t="inlineStr">
@@ -1306,6 +1503,11 @@
         <f>IFERROR(D35/C35,"")</f>
         <v/>
       </c>
+      <c r="F35" s="21" t="n"/>
+      <c r="G35" s="14">
+        <f>IFERROR(F35/C35,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="12" t="inlineStr">
@@ -1329,6 +1531,11 @@
         <f>IFERROR(D36/C36,"")</f>
         <v/>
       </c>
+      <c r="F36" s="21" t="n"/>
+      <c r="G36" s="14">
+        <f>IFERROR(F36/C36,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="12" t="inlineStr">
@@ -1350,6 +1557,11 @@
         <f>IFERROR(D37/C37,"")</f>
         <v>0.9814126394</v>
       </c>
+      <c r="F37" s="21" t="n"/>
+      <c r="G37" s="14">
+        <f>IFERROR(F37/C37,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="12" t="inlineStr">
@@ -1371,6 +1583,11 @@
         <f>IFERROR(D38/C38,"")</f>
         <v>0.96</v>
       </c>
+      <c r="F38" s="21" t="n"/>
+      <c r="G38" s="14">
+        <f>IFERROR(F38/C38,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="12" t="inlineStr">
@@ -1392,6 +1609,13 @@
         <f>IFERROR(D39/C39,"")</f>
         <v>0.652173913</v>
       </c>
+      <c r="F39" s="21" t="n">
+        <v>220000</v>
+      </c>
+      <c r="G39" s="14">
+        <f>IFERROR(F39/C39,"")</f>
+        <v>0.597826087</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="12" t="inlineStr">
@@ -1415,6 +1639,11 @@
         <f>IFERROR(D40/C40,"")</f>
         <v/>
       </c>
+      <c r="F40" s="21" t="n"/>
+      <c r="G40" s="14">
+        <f>IFERROR(F40/C40,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="12" t="inlineStr">
@@ -1438,6 +1667,11 @@
         <f>IFERROR(D41/C41,"")</f>
         <v/>
       </c>
+      <c r="F41" s="21" t="n"/>
+      <c r="G41" s="14">
+        <f>IFERROR(F41/C41,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="12" t="inlineStr">
@@ -1459,6 +1693,11 @@
         <f>IFERROR(D42/C42,"")</f>
         <v>0.9375</v>
       </c>
+      <c r="F42" s="21" t="n"/>
+      <c r="G42" s="14">
+        <f>IFERROR(F42/C42,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="12" t="inlineStr">
@@ -1480,6 +1719,11 @@
         <f>IFERROR(D43/C43,"")</f>
         <v>1.1822660099</v>
       </c>
+      <c r="F43" s="21" t="n"/>
+      <c r="G43" s="14">
+        <f>IFERROR(F43/C43,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="12" t="inlineStr">
@@ -1501,6 +1745,13 @@
         <f>IFERROR(D44/C44,"")</f>
         <v>0.6557377049</v>
       </c>
+      <c r="F44" s="21" t="n">
+        <v>250000</v>
+      </c>
+      <c r="G44" s="14">
+        <f>IFERROR(F44/C44,"")</f>
+        <v>0.6830601093</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="12" t="inlineStr">
@@ -1522,6 +1773,11 @@
         <f>IFERROR(D45/C45,"")</f>
         <v>0.9523809524</v>
       </c>
+      <c r="F45" s="21" t="n"/>
+      <c r="G45" s="14">
+        <f>IFERROR(F45/C45,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="12" t="inlineStr">
@@ -1543,6 +1799,11 @@
         <f>IFERROR(D46/C46,"")</f>
         <v>1.1684210526</v>
       </c>
+      <c r="F46" s="21" t="n"/>
+      <c r="G46" s="14">
+        <f>IFERROR(F46/C46,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="12" t="inlineStr">
@@ -1564,6 +1825,13 @@
         <f>IFERROR(D47/C47,"")</f>
         <v>0.6486486486</v>
       </c>
+      <c r="F47" s="21" t="n">
+        <v>200000</v>
+      </c>
+      <c r="G47" s="14">
+        <f>IFERROR(F47/C47,"")</f>
+        <v>0.6006006006</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="12" t="inlineStr">
@@ -1585,6 +1853,11 @@
         <f>IFERROR(D48/C48,"")</f>
         <v>2.2105263158</v>
       </c>
+      <c r="F48" s="21" t="n"/>
+      <c r="G48" s="14">
+        <f>IFERROR(F48/C48,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="12" t="inlineStr">
@@ -1606,6 +1879,11 @@
         <f>IFERROR(D49/C49,"")</f>
         <v>0.9107142857</v>
       </c>
+      <c r="F49" s="21" t="n"/>
+      <c r="G49" s="14">
+        <f>IFERROR(F49/C49,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="12" t="inlineStr">
@@ -1627,6 +1905,11 @@
         <f>IFERROR(D50/C50,"")</f>
         <v>1.1925465839</v>
       </c>
+      <c r="F50" s="21" t="n"/>
+      <c r="G50" s="14">
+        <f>IFERROR(F50/C50,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="12" t="inlineStr">
@@ -1648,6 +1931,11 @@
         <f>IFERROR(D51/C51,"")</f>
         <v>0.7966804979</v>
       </c>
+      <c r="F51" s="21" t="n"/>
+      <c r="G51" s="14">
+        <f>IFERROR(F51/C51,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="12" t="inlineStr">
@@ -1669,6 +1957,11 @@
         <f>IFERROR(D52/C52,"")</f>
         <v>0.7258064516</v>
       </c>
+      <c r="F52" s="21" t="n"/>
+      <c r="G52" s="14">
+        <f>IFERROR(F52/C52,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="12" t="inlineStr">
@@ -1690,6 +1983,15 @@
         <f>IFERROR(D53/C53,"")</f>
         <v>0.5858585859</v>
       </c>
+      <c r="F53" s="21" t="inlineStr">
+        <is>
+          <t>No offers</t>
+        </is>
+      </c>
+      <c r="G53" s="14">
+        <f>IFERROR(F53/C53,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="12" t="inlineStr">
@@ -1711,6 +2013,11 @@
         <f>IFERROR(D54/C54,"")</f>
         <v>2.0487804878</v>
       </c>
+      <c r="F54" s="21" t="n"/>
+      <c r="G54" s="14">
+        <f>IFERROR(F54/C54,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="12" t="inlineStr">
@@ -1732,6 +2039,13 @@
         <f>IFERROR(D55/C55,"")</f>
         <v>0.4985163205</v>
       </c>
+      <c r="F55" s="21" t="n">
+        <v>160000</v>
+      </c>
+      <c r="G55" s="14">
+        <f>IFERROR(F55/C55,"")</f>
+        <v>0.4747774481</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="12" t="inlineStr">
@@ -1755,6 +2069,11 @@
         <f>IFERROR(D56/C56,"")</f>
         <v/>
       </c>
+      <c r="F56" s="21" t="n"/>
+      <c r="G56" s="14">
+        <f>IFERROR(F56/C56,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="12" t="inlineStr">
@@ -1776,6 +2095,11 @@
         <f>IFERROR(D57/C57,"")</f>
         <v>0.8387096774</v>
       </c>
+      <c r="F57" s="21" t="n"/>
+      <c r="G57" s="14">
+        <f>IFERROR(F57/C57,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="12" t="inlineStr">
@@ -1797,6 +2121,11 @@
         <f>IFERROR(D58/C58,"")</f>
         <v>0.7586206897</v>
       </c>
+      <c r="F58" s="21" t="n"/>
+      <c r="G58" s="14">
+        <f>IFERROR(F58/C58,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="12" t="inlineStr">
@@ -1818,6 +2147,11 @@
         <f>IFERROR(D59/C59,"")</f>
         <v>0.9836065574</v>
       </c>
+      <c r="F59" s="21" t="n"/>
+      <c r="G59" s="14">
+        <f>IFERROR(F59/C59,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="12" t="inlineStr">
@@ -1839,6 +2173,13 @@
         <f>IFERROR(D60/C60,"")</f>
         <v>0.3973509934</v>
       </c>
+      <c r="F60" s="21" t="n">
+        <v>110000</v>
+      </c>
+      <c r="G60" s="14">
+        <f>IFERROR(F60/C60,"")</f>
+        <v>0.3642384106</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="12" t="inlineStr">
@@ -1860,6 +2201,13 @@
         <f>IFERROR(D61/C61,"")</f>
         <v>0.5504587156</v>
       </c>
+      <c r="F61" s="21" t="n">
+        <v>110000</v>
+      </c>
+      <c r="G61" s="14">
+        <f>IFERROR(F61/C61,"")</f>
+        <v>0.504587156</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="12" t="inlineStr">
@@ -1883,6 +2231,11 @@
         <f>IFERROR(D62/C62,"")</f>
         <v/>
       </c>
+      <c r="F62" s="21" t="n"/>
+      <c r="G62" s="14">
+        <f>IFERROR(F62/C62,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="12" t="inlineStr">
@@ -1906,6 +2259,11 @@
         <f>IFERROR(D63/C63,"")</f>
         <v/>
       </c>
+      <c r="F63" s="21" t="n"/>
+      <c r="G63" s="14">
+        <f>IFERROR(F63/C63,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="12" t="inlineStr">
@@ -1929,6 +2287,11 @@
         <f>IFERROR(D64/C64,"")</f>
         <v/>
       </c>
+      <c r="F64" s="21" t="n"/>
+      <c r="G64" s="14">
+        <f>IFERROR(F64/C64,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="12" t="inlineStr">
@@ -1950,6 +2313,13 @@
         <f>IFERROR(D65/C65,"")</f>
         <v>0.456</v>
       </c>
+      <c r="F65" s="21" t="n">
+        <v>145000</v>
+      </c>
+      <c r="G65" s="14">
+        <f>IFERROR(F65/C65,"")</f>
+        <v>0.58</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="12" t="inlineStr">
@@ -1971,6 +2341,15 @@
         <f>IFERROR(D66/C66,"")</f>
         <v>0.6404494382</v>
       </c>
+      <c r="F66" s="21" t="inlineStr">
+        <is>
+          <t>No offers</t>
+        </is>
+      </c>
+      <c r="G66" s="14">
+        <f>IFERROR(F66/C66,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="12" t="inlineStr">
@@ -1992,6 +2371,15 @@
         <f>IFERROR(D67/C67,"")</f>
         <v>0.3149171271</v>
       </c>
+      <c r="F67" s="21" t="inlineStr">
+        <is>
+          <t>No offers</t>
+        </is>
+      </c>
+      <c r="G67" s="14">
+        <f>IFERROR(F67/C67,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="12" t="inlineStr">
@@ -2013,6 +2401,13 @@
         <f>IFERROR(D68/C68,"")</f>
         <v>0.5595854922</v>
       </c>
+      <c r="F68" s="21" t="n">
+        <v>120000</v>
+      </c>
+      <c r="G68" s="14">
+        <f>IFERROR(F68/C68,"")</f>
+        <v>0.621761658</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="12" t="inlineStr">
@@ -2034,6 +2429,13 @@
         <f>IFERROR(D69/C69,"")</f>
         <v>0.5882352941</v>
       </c>
+      <c r="F69" s="21" t="n">
+        <v>75000</v>
+      </c>
+      <c r="G69" s="14">
+        <f>IFERROR(F69/C69,"")</f>
+        <v>0.4901960784</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="12" t="inlineStr">
@@ -2055,6 +2457,13 @@
         <f>IFERROR(D70/C70,"")</f>
         <v>0.6511627907</v>
       </c>
+      <c r="F70" s="21" t="n">
+        <v>115000</v>
+      </c>
+      <c r="G70" s="14">
+        <f>IFERROR(F70/C70,"")</f>
+        <v>0.8914728682</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="12" t="inlineStr">
@@ -2076,6 +2485,13 @@
         <f>IFERROR(D71/C71,"")</f>
         <v>0.4832214765</v>
       </c>
+      <c r="F71" s="21" t="n">
+        <v>75000</v>
+      </c>
+      <c r="G71" s="14">
+        <f>IFERROR(F71/C71,"")</f>
+        <v>0.5033557047</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="12" t="inlineStr">
@@ -2099,6 +2515,11 @@
         <f>IFERROR(D72/C72,"")</f>
         <v/>
       </c>
+      <c r="F72" s="21" t="n"/>
+      <c r="G72" s="14">
+        <f>IFERROR(F72/C72,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="12" t="inlineStr">
@@ -2120,6 +2541,11 @@
         <f>IFERROR(D73/C73,"")</f>
         <v>0.7317073171</v>
       </c>
+      <c r="F73" s="21" t="n"/>
+      <c r="G73" s="14">
+        <f>IFERROR(F73/C73,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="12" t="inlineStr">
@@ -2141,6 +2567,13 @@
         <f>IFERROR(D74/C74,"")</f>
         <v>0.1583113456</v>
       </c>
+      <c r="F74" s="21" t="n">
+        <v>175000</v>
+      </c>
+      <c r="G74" s="14">
+        <f>IFERROR(F74/C74,"")</f>
+        <v>0.4617414248</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="12" t="inlineStr">
@@ -2164,6 +2597,11 @@
         <f>IFERROR(D75/C75,"")</f>
         <v/>
       </c>
+      <c r="F75" s="21" t="n"/>
+      <c r="G75" s="14">
+        <f>IFERROR(F75/C75,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="12" t="inlineStr">
@@ -2185,6 +2623,13 @@
         <f>IFERROR(D76/C76,"")</f>
         <v>0.4615384615</v>
       </c>
+      <c r="F76" s="21" t="n">
+        <v>55000</v>
+      </c>
+      <c r="G76" s="14">
+        <f>IFERROR(F76/C76,"")</f>
+        <v>0.4230769231</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="12" t="inlineStr">
@@ -2206,6 +2651,13 @@
         <f>IFERROR(D77/C77,"")</f>
         <v>0.6171428571</v>
       </c>
+      <c r="F77" s="21" t="n">
+        <v>85000</v>
+      </c>
+      <c r="G77" s="14">
+        <f>IFERROR(F77/C77,"")</f>
+        <v>0.9714285714</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="12" t="inlineStr">
@@ -2227,6 +2679,13 @@
         <f>IFERROR(D78/C78,"")</f>
         <v>0.5189189189</v>
       </c>
+      <c r="F78" s="21" t="n">
+        <v>60000</v>
+      </c>
+      <c r="G78" s="14">
+        <f>IFERROR(F78/C78,"")</f>
+        <v>0.6486486486</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="12" t="inlineStr">
@@ -2250,6 +2709,11 @@
         <f>IFERROR(D79/C79,"")</f>
         <v/>
       </c>
+      <c r="F79" s="21" t="n"/>
+      <c r="G79" s="14">
+        <f>IFERROR(F79/C79,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="12" t="inlineStr">
@@ -2271,6 +2735,13 @@
         <f>IFERROR(D80/C80,"")</f>
         <v>0.4444444444</v>
       </c>
+      <c r="F80" s="21" t="n">
+        <v>55000</v>
+      </c>
+      <c r="G80" s="14">
+        <f>IFERROR(F80/C80,"")</f>
+        <v>0.6790123457</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="12" t="inlineStr">
@@ -2292,6 +2763,11 @@
         <f>IFERROR(D81/C81,"")</f>
         <v>0.9</v>
       </c>
+      <c r="F81" s="21" t="n"/>
+      <c r="G81" s="14">
+        <f>IFERROR(F81/C81,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="12" t="inlineStr">
@@ -2315,6 +2791,11 @@
         <f>IFERROR(D82/C82,"")</f>
         <v/>
       </c>
+      <c r="F82" s="21" t="n"/>
+      <c r="G82" s="14">
+        <f>IFERROR(F82/C82,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="12" t="inlineStr">
@@ -2336,6 +2817,13 @@
         <f>IFERROR(D83/C83,"")</f>
         <v>0.3658536585</v>
       </c>
+      <c r="F83" s="21" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G83" s="14">
+        <f>IFERROR(F83/C83,"")</f>
+        <v>0.6097560976</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="12" t="inlineStr">
@@ -2357,6 +2845,13 @@
         <f>IFERROR(D84/C84,"")</f>
         <v>0.0967741935</v>
       </c>
+      <c r="F84" s="21" t="n">
+        <v>25000</v>
+      </c>
+      <c r="G84" s="14">
+        <f>IFERROR(F84/C84,"")</f>
+        <v>0.0806451613</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="12" t="inlineStr">
@@ -2378,6 +2873,13 @@
         <f>IFERROR(D85/C85,"")</f>
         <v>0.2666666667</v>
       </c>
+      <c r="F85" s="21" t="n">
+        <v>40000</v>
+      </c>
+      <c r="G85" s="14">
+        <f>IFERROR(F85/C85,"")</f>
+        <v>0.4444444444</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="12" t="inlineStr">
@@ -2399,6 +2901,15 @@
         <f>IFERROR(D86/C86,"")</f>
         <v>0.3720930233</v>
       </c>
+      <c r="F86" s="21" t="inlineStr">
+        <is>
+          <t>No offers</t>
+        </is>
+      </c>
+      <c r="G86" s="14">
+        <f>IFERROR(F86/C86,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="12" t="inlineStr">
@@ -2420,6 +2931,13 @@
         <f>IFERROR(D87/C87,"")</f>
         <v>0.2142857143</v>
       </c>
+      <c r="F87" s="21" t="n">
+        <v>30000</v>
+      </c>
+      <c r="G87" s="14">
+        <f>IFERROR(F87/C87,"")</f>
+        <v>0.2678571429</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="12" t="inlineStr">
@@ -2441,6 +2959,13 @@
         <f>IFERROR(D88/C88,"")</f>
         <v>0.1764705882</v>
       </c>
+      <c r="F88" s="21" t="n">
+        <v>45000</v>
+      </c>
+      <c r="G88" s="14">
+        <f>IFERROR(F88/C88,"")</f>
+        <v>0.3308823529</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="12" t="inlineStr">
@@ -2462,6 +2987,11 @@
         <f>IFERROR(D89/C89,"")</f>
         <v>0.8780487805</v>
       </c>
+      <c r="F89" s="21" t="n"/>
+      <c r="G89" s="14">
+        <f>IFERROR(F89/C89,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="12" t="inlineStr">
@@ -2485,6 +3015,11 @@
         <f>IFERROR(D90/C90,"")</f>
         <v/>
       </c>
+      <c r="F90" s="21" t="n"/>
+      <c r="G90" s="14">
+        <f>IFERROR(F90/C90,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="12" t="inlineStr">
@@ -2508,6 +3043,11 @@
         <f>IFERROR(D91/C91,"")</f>
         <v/>
       </c>
+      <c r="F91" s="21" t="n"/>
+      <c r="G91" s="14">
+        <f>IFERROR(F91/C91,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="12" t="inlineStr">
@@ -2531,6 +3071,11 @@
         <f>IFERROR(D92/C92,"")</f>
         <v/>
       </c>
+      <c r="F92" s="21" t="n"/>
+      <c r="G92" s="14">
+        <f>IFERROR(F92/C92,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="12" t="inlineStr">
@@ -2552,6 +3097,13 @@
         <f>IFERROR(D93/C93,"")</f>
         <v>0.04</v>
       </c>
+      <c r="F93" s="21" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G93" s="14">
+        <f>IFERROR(F93/C93,"")</f>
+        <v>0.0333333333</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="12" t="inlineStr">
@@ -2575,6 +3127,11 @@
         <f>IFERROR(D94/C94,"")</f>
         <v/>
       </c>
+      <c r="F94" s="21" t="n"/>
+      <c r="G94" s="14">
+        <f>IFERROR(F94/C94,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="12" t="inlineStr">
@@ -2598,6 +3155,11 @@
         <f>IFERROR(D95/C95,"")</f>
         <v/>
       </c>
+      <c r="F95" s="21" t="n"/>
+      <c r="G95" s="14">
+        <f>IFERROR(F95/C95,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="12" t="inlineStr">
@@ -2621,6 +3183,11 @@
         <f>IFERROR(D96/C96,"")</f>
         <v/>
       </c>
+      <c r="F96" s="21" t="n"/>
+      <c r="G96" s="14">
+        <f>IFERROR(F96/C96,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="12" t="inlineStr">
@@ -2644,6 +3211,11 @@
         <f>IFERROR(D97/C97,"")</f>
         <v/>
       </c>
+      <c r="F97" s="21" t="n"/>
+      <c r="G97" s="14">
+        <f>IFERROR(F97/C97,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="12" t="inlineStr">
@@ -2667,6 +3239,11 @@
         <f>IFERROR(D98/C98,"")</f>
         <v/>
       </c>
+      <c r="F98" s="21" t="n"/>
+      <c r="G98" s="14">
+        <f>IFERROR(F98/C98,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="12" t="inlineStr">
@@ -2690,6 +3267,11 @@
         <f>IFERROR(D99/C99,"")</f>
         <v/>
       </c>
+      <c r="F99" s="21" t="n"/>
+      <c r="G99" s="14">
+        <f>IFERROR(F99/C99,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="12" t="inlineStr">
@@ -2713,6 +3295,11 @@
         <f>IFERROR(D100/C100,"")</f>
         <v/>
       </c>
+      <c r="F100" s="21" t="n"/>
+      <c r="G100" s="14">
+        <f>IFERROR(F100/C100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="12" t="inlineStr">
@@ -2732,9 +3319,14 @@
         <f>IFERROR(D101/C101,"")</f>
         <v/>
       </c>
+      <c r="F101" s="21" t="n"/>
+      <c r="G101" s="14">
+        <f>IFERROR(F101/C101,"")</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E101"/>
+  <autoFilter ref="A1:G101"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8632,7 +9224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A72"/>
+  <dimension ref="A1:A82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -9088,6 +9680,69 @@
         </is>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" s="23" t="inlineStr">
+        <is>
+          <t>Offer likely accepted</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="24" t="inlineStr">
+        <is>
+          <t>Carried from the 'Offer likely accepted (£)' column of the source spreadsheet: 26 lots have</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="24" t="inlineStr">
+        <is>
+          <t>a figure, 7 are marked 'No offers' (that is a recorded result, not a gap), and 67 are blank</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="24" t="inlineStr">
+        <is>
+          <t>because no offer was pursued.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="24" t="inlineStr">
+        <is>
+          <t>These offers relate to the SEPTEMBER sale. Where a lot has been re-entered in October at a cut</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="24" t="inlineStr">
+        <is>
+          <t>guide, the offer may no longer reflect the market - lot 166 (New Bank House) is the clearest</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="24" t="inlineStr">
+        <is>
+          <t>case, offer £35,000 against an October guide of £5,000-£15,000.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="24" t="inlineStr">
+        <is>
+          <t>'Offer as % of Hometrack' is the offer divided by the Hometrack valuation, on the same caution</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="24" t="inlineStr">
+        <is>
+          <t>as the guide+20% comparison: over 100% usually means a bad AVM match, not an overpayment.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add October catalogue sheet, built from the website list
The workbook was organised around our September spreadsheet, asking which
of those lots resurfaced. This adds the inverse and makes it the first
sheet: all 93 lots from the auction house's current-auction page, which is
the list of what is actually on offer.

Each row carries guide, guide +20%, and - where we already hold them from
September - Hometrack, accepted offer and Serco status, with a column
saying whether the lot is one we have seen before or is new to us.

The gap this exposes is the point of the sheet: only 7 of 93 lots have a
Hometrack figure, because 80 are lots we have never valued. Those need
pulling from Sourcing Brain before the October sale can be worked properly.

Cached values re-patched across all three sheets (400 cells, verified).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Kgh51upqvBx4um6iPVc7Lf
</commit_message>
<xml_diff>
--- a/auction_xref/Auction lots - checked list.xlsx
+++ b/auction_xref/Auction lots - checked list.xlsx
@@ -7,13 +7,15 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Working list" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Checked list" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Notes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="October catalogue" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Working list" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Checked list" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Notes" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Working list'!$A$1:$G$101</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Checked list'!$A$1:$O$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'October catalogue'!$A$1:$I$94</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Working list'!$A$1:$G$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Checked list'!$A$1:$O$101</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -103,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -173,6 +175,33 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -538,6 +567,3046 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I94"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Oct lot</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Guide price</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Guide +20%</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Hometrack valuation</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Guide +20% as % of Hometrack</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Offer likely accepted (£)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Serco status</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Seen in September?</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>72 Ibsley Gardens, Wandsworth, London, SW15 4JW</t>
+        </is>
+      </c>
+      <c r="C2" s="26" t="n">
+        <v>290000</v>
+      </c>
+      <c r="D2" s="26">
+        <f>IFERROR(C2*1.2,"")</f>
+        <v>348000.0</v>
+      </c>
+      <c r="E2" s="25" t="n"/>
+      <c r="F2" s="27">
+        <f>IFERROR(D2/E2,"")</f>
+        <v/>
+      </c>
+      <c r="G2" s="25" t="n"/>
+      <c r="H2" s="25" t="n"/>
+      <c r="I2" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="25" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>24 Timsbury Walk, Wandsworth, London, SW15 4LN</t>
+        </is>
+      </c>
+      <c r="C3" s="26" t="n">
+        <v>290000</v>
+      </c>
+      <c r="D3" s="26">
+        <f>IFERROR(C3*1.2,"")</f>
+        <v>348000.0</v>
+      </c>
+      <c r="E3" s="25" t="n"/>
+      <c r="F3" s="27">
+        <f>IFERROR(D3/E3,"")</f>
+        <v/>
+      </c>
+      <c r="G3" s="25" t="n"/>
+      <c r="H3" s="25" t="n"/>
+      <c r="I3" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="25" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>80 Flintmill Crescent, Blackheath, London, SE3 8LY</t>
+        </is>
+      </c>
+      <c r="C4" s="26" t="n">
+        <v>140000</v>
+      </c>
+      <c r="D4" s="26">
+        <f>IFERROR(C4*1.2,"")</f>
+        <v>168000.0</v>
+      </c>
+      <c r="E4" s="25" t="n"/>
+      <c r="F4" s="27">
+        <f>IFERROR(D4/E4,"")</f>
+        <v/>
+      </c>
+      <c r="G4" s="25" t="n"/>
+      <c r="H4" s="25" t="n"/>
+      <c r="I4" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="25" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>Apartment 404 Weymouth Building, 2 Deacon Street, Elephant &amp; Castle, London, SE17 1GB</t>
+        </is>
+      </c>
+      <c r="C5" s="26" t="n">
+        <v>410000</v>
+      </c>
+      <c r="D5" s="26">
+        <f>IFERROR(C5*1.2,"")</f>
+        <v>492000.0</v>
+      </c>
+      <c r="E5" s="25" t="n"/>
+      <c r="F5" s="27">
+        <f>IFERROR(D5/E5,"")</f>
+        <v/>
+      </c>
+      <c r="G5" s="25" t="n"/>
+      <c r="H5" s="25" t="n"/>
+      <c r="I5" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="25" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>62 Crowther Road, South Norwood, London, SE25 5QP</t>
+        </is>
+      </c>
+      <c r="C6" s="26" t="n">
+        <v>160000</v>
+      </c>
+      <c r="D6" s="26">
+        <f>IFERROR(C6*1.2,"")</f>
+        <v>192000.0</v>
+      </c>
+      <c r="E6" s="25" t="n"/>
+      <c r="F6" s="27">
+        <f>IFERROR(D6/E6,"")</f>
+        <v/>
+      </c>
+      <c r="G6" s="25" t="n"/>
+      <c r="H6" s="25" t="n"/>
+      <c r="I6" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="25" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>18 Toronto Avenue, Manor Park, London, E12 5JF</t>
+        </is>
+      </c>
+      <c r="C7" s="26" t="n">
+        <v>300000</v>
+      </c>
+      <c r="D7" s="26">
+        <f>IFERROR(C7*1.2,"")</f>
+        <v>360000.0</v>
+      </c>
+      <c r="E7" s="25" t="n"/>
+      <c r="F7" s="27">
+        <f>IFERROR(D7/E7,"")</f>
+        <v/>
+      </c>
+      <c r="G7" s="25" t="n"/>
+      <c r="H7" s="25" t="n"/>
+      <c r="I7" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="25" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>51 Hendon Way, Cricklewood, London, NW2 2LX</t>
+        </is>
+      </c>
+      <c r="C8" s="26" t="n">
+        <v>625000</v>
+      </c>
+      <c r="D8" s="26">
+        <f>IFERROR(C8*1.2,"")</f>
+        <v>750000.0</v>
+      </c>
+      <c r="E8" s="25" t="n"/>
+      <c r="F8" s="27">
+        <f>IFERROR(D8/E8,"")</f>
+        <v/>
+      </c>
+      <c r="G8" s="25" t="n"/>
+      <c r="H8" s="25" t="n"/>
+      <c r="I8" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="25" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>177 Morley Avenue, Wood Green, London, N22 6NT</t>
+        </is>
+      </c>
+      <c r="C9" s="26" t="n">
+        <v>385000</v>
+      </c>
+      <c r="D9" s="26">
+        <f>IFERROR(C9*1.2,"")</f>
+        <v>462000.0</v>
+      </c>
+      <c r="E9" s="25" t="n"/>
+      <c r="F9" s="27">
+        <f>IFERROR(D9/E9,"")</f>
+        <v/>
+      </c>
+      <c r="G9" s="25" t="n"/>
+      <c r="H9" s="25" t="n"/>
+      <c r="I9" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="25" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>115 Stoke Newington Road, Stoke Newington, London, N16 8BX</t>
+        </is>
+      </c>
+      <c r="C10" s="26" t="n">
+        <v>250000</v>
+      </c>
+      <c r="D10" s="26">
+        <f>IFERROR(C10*1.2,"")</f>
+        <v>300000.0</v>
+      </c>
+      <c r="E10" s="25" t="n"/>
+      <c r="F10" s="27">
+        <f>IFERROR(D10/E10,"")</f>
+        <v/>
+      </c>
+      <c r="G10" s="25" t="n"/>
+      <c r="H10" s="25" t="n"/>
+      <c r="I10" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="25" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>Flat 6, 317 Barking Road, Plaistow, London, E13 8EE</t>
+        </is>
+      </c>
+      <c r="C11" s="26" t="n">
+        <v>100000</v>
+      </c>
+      <c r="D11" s="26">
+        <f>IFERROR(C11*1.2,"")</f>
+        <v>120000.0</v>
+      </c>
+      <c r="E11" s="25" t="n"/>
+      <c r="F11" s="27">
+        <f>IFERROR(D11/E11,"")</f>
+        <v/>
+      </c>
+      <c r="G11" s="25" t="n"/>
+      <c r="H11" s="25" t="n"/>
+      <c r="I11" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="25" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>24 Macquarie Way, Isle of Dogs, London, E14 3AU</t>
+        </is>
+      </c>
+      <c r="C12" s="26" t="n">
+        <v>700000</v>
+      </c>
+      <c r="D12" s="26">
+        <f>IFERROR(C12*1.2,"")</f>
+        <v>840000.0</v>
+      </c>
+      <c r="E12" s="25" t="n"/>
+      <c r="F12" s="27">
+        <f>IFERROR(D12/E12,"")</f>
+        <v/>
+      </c>
+      <c r="G12" s="25" t="n"/>
+      <c r="H12" s="25" t="n"/>
+      <c r="I12" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="25" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>23 Hale End Road, Walthamstow, London, E17 4BG</t>
+        </is>
+      </c>
+      <c r="C13" s="26" t="n">
+        <v>370000</v>
+      </c>
+      <c r="D13" s="26">
+        <f>IFERROR(C13*1.2,"")</f>
+        <v>444000.0</v>
+      </c>
+      <c r="E13" s="25" t="n"/>
+      <c r="F13" s="27">
+        <f>IFERROR(D13/E13,"")</f>
+        <v/>
+      </c>
+      <c r="G13" s="25" t="n"/>
+      <c r="H13" s="25" t="n"/>
+      <c r="I13" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="25" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>38 Gunnersbury Avenue, Acton, London, W5 4HA</t>
+        </is>
+      </c>
+      <c r="C14" s="26" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="D14" s="26">
+        <f>IFERROR(C14*1.2,"")</f>
+        <v>1440000.0</v>
+      </c>
+      <c r="E14" s="25" t="n"/>
+      <c r="F14" s="27">
+        <f>IFERROR(D14/E14,"")</f>
+        <v/>
+      </c>
+      <c r="G14" s="25" t="n"/>
+      <c r="H14" s="25" t="n"/>
+      <c r="I14" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="25" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>Flat 54, 105 Hallam Street, Marylebone, London, W1W 5HE</t>
+        </is>
+      </c>
+      <c r="C15" s="26" t="n">
+        <v>200000</v>
+      </c>
+      <c r="D15" s="26">
+        <f>IFERROR(C15*1.2,"")</f>
+        <v>240000.0</v>
+      </c>
+      <c r="E15" s="25" t="n"/>
+      <c r="F15" s="27">
+        <f>IFERROR(D15/E15,"")</f>
+        <v/>
+      </c>
+      <c r="G15" s="25" t="n"/>
+      <c r="H15" s="25" t="n"/>
+      <c r="I15" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="25" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Flat 15 Cobden Court, Byron Close, Greenwich, London, SE28 8AG</t>
+        </is>
+      </c>
+      <c r="C16" s="26" t="n">
+        <v>150000</v>
+      </c>
+      <c r="D16" s="26">
+        <f>IFERROR(C16*1.2,"")</f>
+        <v>180000.0</v>
+      </c>
+      <c r="E16" s="25" t="n"/>
+      <c r="F16" s="27">
+        <f>IFERROR(D16/E16,"")</f>
+        <v/>
+      </c>
+      <c r="G16" s="25" t="n"/>
+      <c r="H16" s="25" t="n"/>
+      <c r="I16" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="25" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>Flat 2, 69 Johnson Street, Shadwell, London, E1 0AQ</t>
+        </is>
+      </c>
+      <c r="C17" s="26" t="n">
+        <v>275000</v>
+      </c>
+      <c r="D17" s="26">
+        <f>IFERROR(C17*1.2,"")</f>
+        <v>330000.0</v>
+      </c>
+      <c r="E17" s="25" t="n"/>
+      <c r="F17" s="27">
+        <f>IFERROR(D17/E17,"")</f>
+        <v/>
+      </c>
+      <c r="G17" s="25" t="n"/>
+      <c r="H17" s="25" t="n"/>
+      <c r="I17" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="25" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>316B Lordship Lane, East Dulwich, London, SE22 8LY</t>
+        </is>
+      </c>
+      <c r="C18" s="26" t="n">
+        <v>390000</v>
+      </c>
+      <c r="D18" s="26">
+        <f>IFERROR(C18*1.2,"")</f>
+        <v>468000.0</v>
+      </c>
+      <c r="E18" s="25" t="n"/>
+      <c r="F18" s="27">
+        <f>IFERROR(D18/E18,"")</f>
+        <v/>
+      </c>
+      <c r="G18" s="25" t="n"/>
+      <c r="H18" s="25" t="n"/>
+      <c r="I18" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="25" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>5 Guild House, 393 Rotherhithe New Road, Bermondsey, London, SE16 3FN</t>
+        </is>
+      </c>
+      <c r="C19" s="26" t="n">
+        <v>310000</v>
+      </c>
+      <c r="D19" s="26">
+        <f>IFERROR(C19*1.2,"")</f>
+        <v>372000.0</v>
+      </c>
+      <c r="E19" s="25" t="n"/>
+      <c r="F19" s="27">
+        <f>IFERROR(D19/E19,"")</f>
+        <v/>
+      </c>
+      <c r="G19" s="25" t="n"/>
+      <c r="H19" s="25" t="n"/>
+      <c r="I19" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="25" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>20A Hayland Close, Kingsbury, London, NW9 0LH</t>
+        </is>
+      </c>
+      <c r="C20" s="26" t="n">
+        <v>225000</v>
+      </c>
+      <c r="D20" s="26">
+        <f>IFERROR(C20*1.2,"")</f>
+        <v>270000.0</v>
+      </c>
+      <c r="E20" s="25" t="n"/>
+      <c r="F20" s="27">
+        <f>IFERROR(D20/E20,"")</f>
+        <v/>
+      </c>
+      <c r="G20" s="25" t="n"/>
+      <c r="H20" s="25" t="n"/>
+      <c r="I20" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="28" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Flat 11 Regatta Point, 1 Manilla Street, Canary Wharf, London, E14 8JZ</t>
+        </is>
+      </c>
+      <c r="C21" s="29" t="n">
+        <v>180000</v>
+      </c>
+      <c r="D21" s="29">
+        <f>IFERROR(C21*1.2,"")</f>
+        <v>216000.0</v>
+      </c>
+      <c r="E21" s="29" t="n">
+        <v>303000</v>
+      </c>
+      <c r="F21" s="30">
+        <f>IFERROR(D21/E21,"")</f>
+        <v>0.7128712871</v>
+      </c>
+      <c r="G21" s="28" t="n"/>
+      <c r="H21" s="28" t="inlineStr">
+        <is>
+          <t>Outside region</t>
+        </is>
+      </c>
+      <c r="I21" s="28" t="inlineStr">
+        <is>
+          <t>Yes - Sept lot 94</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="28" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Flat 3 Regatta Point, 1 Manilla Street, Canary Wharf, London, E14 8JZ</t>
+        </is>
+      </c>
+      <c r="C22" s="29" t="n">
+        <v>225000</v>
+      </c>
+      <c r="D22" s="29">
+        <f>IFERROR(C22*1.2,"")</f>
+        <v>270000.0</v>
+      </c>
+      <c r="E22" s="29" t="n">
+        <v>370000</v>
+      </c>
+      <c r="F22" s="30">
+        <f>IFERROR(D22/E22,"")</f>
+        <v>0.7297297297</v>
+      </c>
+      <c r="G22" s="28" t="n"/>
+      <c r="H22" s="28" t="inlineStr">
+        <is>
+          <t>Outside region</t>
+        </is>
+      </c>
+      <c r="I22" s="28" t="inlineStr">
+        <is>
+          <t>Yes - Sept lot 95</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="25" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>Flat 2, 3 Cottage Road, Highbury, London, N7 8TP</t>
+        </is>
+      </c>
+      <c r="C23" s="26" t="n">
+        <v>395000</v>
+      </c>
+      <c r="D23" s="26">
+        <f>IFERROR(C23*1.2,"")</f>
+        <v>474000.0</v>
+      </c>
+      <c r="E23" s="25" t="n"/>
+      <c r="F23" s="27">
+        <f>IFERROR(D23/E23,"")</f>
+        <v/>
+      </c>
+      <c r="G23" s="25" t="n"/>
+      <c r="H23" s="25" t="n"/>
+      <c r="I23" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="25" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>4 Swansea Court, Beckton, London, E16 2RT</t>
+        </is>
+      </c>
+      <c r="C24" s="26" t="n">
+        <v>150000</v>
+      </c>
+      <c r="D24" s="26">
+        <f>IFERROR(C24*1.2,"")</f>
+        <v>180000.0</v>
+      </c>
+      <c r="E24" s="25" t="n"/>
+      <c r="F24" s="27">
+        <f>IFERROR(D24/E24,"")</f>
+        <v/>
+      </c>
+      <c r="G24" s="25" t="n"/>
+      <c r="H24" s="25" t="n"/>
+      <c r="I24" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="25" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>Flat D, 49 High Street, Penge, London, SE20 7HW</t>
+        </is>
+      </c>
+      <c r="C25" s="26" t="n">
+        <v>85000</v>
+      </c>
+      <c r="D25" s="26">
+        <f>IFERROR(C25*1.2,"")</f>
+        <v>102000.0</v>
+      </c>
+      <c r="E25" s="25" t="n"/>
+      <c r="F25" s="27">
+        <f>IFERROR(D25/E25,"")</f>
+        <v/>
+      </c>
+      <c r="G25" s="25" t="n"/>
+      <c r="H25" s="25" t="n"/>
+      <c r="I25" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="25" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>Flat 40 Weston Court, 4 Brindley Place, Uxbridge, Middlesex, UB8 2UF</t>
+        </is>
+      </c>
+      <c r="C26" s="26" t="n">
+        <v>280000</v>
+      </c>
+      <c r="D26" s="26">
+        <f>IFERROR(C26*1.2,"")</f>
+        <v>336000.0</v>
+      </c>
+      <c r="E26" s="25" t="n"/>
+      <c r="F26" s="27">
+        <f>IFERROR(D26/E26,"")</f>
+        <v/>
+      </c>
+      <c r="G26" s="25" t="n"/>
+      <c r="H26" s="25" t="n"/>
+      <c r="I26" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="25" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>28 Norfolk Road, Thornton Heath, Croydon, CR7 8ND</t>
+        </is>
+      </c>
+      <c r="C27" s="26" t="n">
+        <v>40000</v>
+      </c>
+      <c r="D27" s="26">
+        <f>IFERROR(C27*1.2,"")</f>
+        <v>48000.0</v>
+      </c>
+      <c r="E27" s="25" t="n"/>
+      <c r="F27" s="27">
+        <f>IFERROR(D27/E27,"")</f>
+        <v/>
+      </c>
+      <c r="G27" s="25" t="n"/>
+      <c r="H27" s="25" t="n"/>
+      <c r="I27" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="31" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>105 Highland Road, Bromley, Kent, BR1 4AA</t>
+        </is>
+      </c>
+      <c r="C28" s="31" t="n"/>
+      <c r="D28" s="32">
+        <f>IFERROR(C28*1.2,"")</f>
+        <v/>
+      </c>
+      <c r="E28" s="31" t="n"/>
+      <c r="F28" s="33">
+        <f>IFERROR(D28/E28,"")</f>
+        <v/>
+      </c>
+      <c r="G28" s="31" t="n"/>
+      <c r="H28" s="31" t="n"/>
+      <c r="I28" s="31" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="25" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>Flat 11 Hartsbourne Park, 180 High Road, Bushey Heath, Bushey, Hertfordshire, WD23 1SD</t>
+        </is>
+      </c>
+      <c r="C29" s="26" t="n">
+        <v>550000</v>
+      </c>
+      <c r="D29" s="26">
+        <f>IFERROR(C29*1.2,"")</f>
+        <v>660000.0</v>
+      </c>
+      <c r="E29" s="25" t="n"/>
+      <c r="F29" s="27">
+        <f>IFERROR(D29/E29,"")</f>
+        <v/>
+      </c>
+      <c r="G29" s="25" t="n"/>
+      <c r="H29" s="25" t="n"/>
+      <c r="I29" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="25" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>Flat 304 Platinum House, Lyon Road, Harrow, Middlesex, HA1 2EX</t>
+        </is>
+      </c>
+      <c r="C30" s="26" t="n">
+        <v>160000</v>
+      </c>
+      <c r="D30" s="26">
+        <f>IFERROR(C30*1.2,"")</f>
+        <v>192000.0</v>
+      </c>
+      <c r="E30" s="25" t="n"/>
+      <c r="F30" s="27">
+        <f>IFERROR(D30/E30,"")</f>
+        <v/>
+      </c>
+      <c r="G30" s="25" t="n"/>
+      <c r="H30" s="25" t="n"/>
+      <c r="I30" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="25" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>Flat 12 Arliss Court, 24 Clarendon Road, Watford, Hertfordshire, WD17 1JY</t>
+        </is>
+      </c>
+      <c r="C31" s="26" t="n">
+        <v>180000</v>
+      </c>
+      <c r="D31" s="26">
+        <f>IFERROR(C31*1.2,"")</f>
+        <v>216000.0</v>
+      </c>
+      <c r="E31" s="25" t="n"/>
+      <c r="F31" s="27">
+        <f>IFERROR(D31/E31,"")</f>
+        <v/>
+      </c>
+      <c r="G31" s="25" t="n"/>
+      <c r="H31" s="25" t="n"/>
+      <c r="I31" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="28" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>2102 Kew Eye Apartments, Ealing Road, Brentford, Middlesex, TW8 0GA</t>
+        </is>
+      </c>
+      <c r="C32" s="29" t="n">
+        <v>410000</v>
+      </c>
+      <c r="D32" s="29">
+        <f>IFERROR(C32*1.2,"")</f>
+        <v>492000.0</v>
+      </c>
+      <c r="E32" s="29" t="n">
+        <v>499000</v>
+      </c>
+      <c r="F32" s="30">
+        <f>IFERROR(D32/E32,"")</f>
+        <v>0.9859719439</v>
+      </c>
+      <c r="G32" s="28" t="n"/>
+      <c r="H32" s="28" t="inlineStr">
+        <is>
+          <t>Outside region</t>
+        </is>
+      </c>
+      <c r="I32" s="28" t="inlineStr">
+        <is>
+          <t>Yes - Sept lot 153</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="25" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>Flat 27 Hemingford Court, Gartlet Road, Watford, Hertfordshire, WD17 2AQ</t>
+        </is>
+      </c>
+      <c r="C33" s="26" t="n">
+        <v>175000</v>
+      </c>
+      <c r="D33" s="26">
+        <f>IFERROR(C33*1.2,"")</f>
+        <v>210000.0</v>
+      </c>
+      <c r="E33" s="25" t="n"/>
+      <c r="F33" s="27">
+        <f>IFERROR(D33/E33,"")</f>
+        <v/>
+      </c>
+      <c r="G33" s="25" t="n"/>
+      <c r="H33" s="25" t="n"/>
+      <c r="I33" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="28" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>10 Eider Close, Hayes, Middlesex, UB4 9TD</t>
+        </is>
+      </c>
+      <c r="C34" s="29" t="n">
+        <v>395000</v>
+      </c>
+      <c r="D34" s="29">
+        <f>IFERROR(C34*1.2,"")</f>
+        <v>474000.0</v>
+      </c>
+      <c r="E34" s="29" t="n">
+        <v>458000</v>
+      </c>
+      <c r="F34" s="30">
+        <f>IFERROR(D34/E34,"")</f>
+        <v>1.0349344978</v>
+      </c>
+      <c r="G34" s="28" t="n"/>
+      <c r="H34" s="28" t="inlineStr">
+        <is>
+          <t>Outside region</t>
+        </is>
+      </c>
+      <c r="I34" s="28" t="inlineStr">
+        <is>
+          <t>Yes - Sept lot 92</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="25" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>165A Darkes Lane, Potters Bar, Hertfordshire, EN6 1BW</t>
+        </is>
+      </c>
+      <c r="C35" s="26" t="n">
+        <v>350000</v>
+      </c>
+      <c r="D35" s="26">
+        <f>IFERROR(C35*1.2,"")</f>
+        <v>420000.0</v>
+      </c>
+      <c r="E35" s="25" t="n"/>
+      <c r="F35" s="27">
+        <f>IFERROR(D35/E35,"")</f>
+        <v/>
+      </c>
+      <c r="G35" s="25" t="n"/>
+      <c r="H35" s="25" t="n"/>
+      <c r="I35" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="25" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>41 Oakhall Court, Oakhall Drive, Sunbury-on-Thames, Middlesex, TW16 7LE</t>
+        </is>
+      </c>
+      <c r="C36" s="26" t="n">
+        <v>140000</v>
+      </c>
+      <c r="D36" s="26">
+        <f>IFERROR(C36*1.2,"")</f>
+        <v>168000.0</v>
+      </c>
+      <c r="E36" s="25" t="n"/>
+      <c r="F36" s="27">
+        <f>IFERROR(D36/E36,"")</f>
+        <v/>
+      </c>
+      <c r="G36" s="25" t="n"/>
+      <c r="H36" s="25" t="n"/>
+      <c r="I36" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="25" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>Flat 13 Lexington House, 35 Park Lodge Avenue, West Drayton, Hillingdon, UB7 9FJ</t>
+        </is>
+      </c>
+      <c r="C37" s="26" t="n">
+        <v>150000</v>
+      </c>
+      <c r="D37" s="26">
+        <f>IFERROR(C37*1.2,"")</f>
+        <v>180000.0</v>
+      </c>
+      <c r="E37" s="25" t="n"/>
+      <c r="F37" s="27">
+        <f>IFERROR(D37/E37,"")</f>
+        <v/>
+      </c>
+      <c r="G37" s="25" t="n"/>
+      <c r="H37" s="25" t="n"/>
+      <c r="I37" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="25" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>Flat 8 Keats House, Porchester Mead, Beckenham, Kent, BR3 1TD</t>
+        </is>
+      </c>
+      <c r="C38" s="26" t="n">
+        <v>155000</v>
+      </c>
+      <c r="D38" s="26">
+        <f>IFERROR(C38*1.2,"")</f>
+        <v>186000.0</v>
+      </c>
+      <c r="E38" s="25" t="n"/>
+      <c r="F38" s="27">
+        <f>IFERROR(D38/E38,"")</f>
+        <v/>
+      </c>
+      <c r="G38" s="25" t="n"/>
+      <c r="H38" s="25" t="n"/>
+      <c r="I38" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="25" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>172 Havering Road, Romford, Essex, RM1 4TD</t>
+        </is>
+      </c>
+      <c r="C39" s="26" t="n">
+        <v>270000</v>
+      </c>
+      <c r="D39" s="26">
+        <f>IFERROR(C39*1.2,"")</f>
+        <v>324000.0</v>
+      </c>
+      <c r="E39" s="25" t="n"/>
+      <c r="F39" s="27">
+        <f>IFERROR(D39/E39,"")</f>
+        <v/>
+      </c>
+      <c r="G39" s="25" t="n"/>
+      <c r="H39" s="25" t="n"/>
+      <c r="I39" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="25" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>6A St. Edwards Way, Romford, Essex, RM1 4DD</t>
+        </is>
+      </c>
+      <c r="C40" s="26" t="n">
+        <v>110000</v>
+      </c>
+      <c r="D40" s="26">
+        <f>IFERROR(C40*1.2,"")</f>
+        <v>132000.0</v>
+      </c>
+      <c r="E40" s="25" t="n"/>
+      <c r="F40" s="27">
+        <f>IFERROR(D40/E40,"")</f>
+        <v/>
+      </c>
+      <c r="G40" s="25" t="n"/>
+      <c r="H40" s="25" t="n"/>
+      <c r="I40" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="25" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>Flat 41 Ashcroft Place, Epsom Road, Leatherhead, Surrey, KT22 8RJ</t>
+        </is>
+      </c>
+      <c r="C41" s="26" t="n">
+        <v>130000</v>
+      </c>
+      <c r="D41" s="26">
+        <f>IFERROR(C41*1.2,"")</f>
+        <v>156000.0</v>
+      </c>
+      <c r="E41" s="25" t="n"/>
+      <c r="F41" s="27">
+        <f>IFERROR(D41/E41,"")</f>
+        <v/>
+      </c>
+      <c r="G41" s="25" t="n"/>
+      <c r="H41" s="25" t="n"/>
+      <c r="I41" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="25" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>Flat 2 Burniston Court, 90 Manor Road, Wallington, Surrey, SM6 0AD</t>
+        </is>
+      </c>
+      <c r="C42" s="26" t="n">
+        <v>65000</v>
+      </c>
+      <c r="D42" s="26">
+        <f>IFERROR(C42*1.2,"")</f>
+        <v>78000.0</v>
+      </c>
+      <c r="E42" s="25" t="n"/>
+      <c r="F42" s="27">
+        <f>IFERROR(D42/E42,"")</f>
+        <v/>
+      </c>
+      <c r="G42" s="25" t="n"/>
+      <c r="H42" s="25" t="n"/>
+      <c r="I42" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="25" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>Flat 8, 390 London Road, Croydon, Surrey, CR0 2SW</t>
+        </is>
+      </c>
+      <c r="C43" s="26" t="n">
+        <v>105000</v>
+      </c>
+      <c r="D43" s="26">
+        <f>IFERROR(C43*1.2,"")</f>
+        <v>126000.0</v>
+      </c>
+      <c r="E43" s="25" t="n"/>
+      <c r="F43" s="27">
+        <f>IFERROR(D43/E43,"")</f>
+        <v/>
+      </c>
+      <c r="G43" s="25" t="n"/>
+      <c r="H43" s="25" t="n"/>
+      <c r="I43" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="25" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>11A Windmill Road, Croydon, Surrey, CR0 2XR</t>
+        </is>
+      </c>
+      <c r="C44" s="26" t="n">
+        <v>140000</v>
+      </c>
+      <c r="D44" s="26">
+        <f>IFERROR(C44*1.2,"")</f>
+        <v>168000.0</v>
+      </c>
+      <c r="E44" s="25" t="n"/>
+      <c r="F44" s="27">
+        <f>IFERROR(D44/E44,"")</f>
+        <v/>
+      </c>
+      <c r="G44" s="25" t="n"/>
+      <c r="H44" s="25" t="n"/>
+      <c r="I44" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="25" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>Flat 53 Longitude Apartments, 7 Addiscombe Grove, Croydon, Surrey, CR0 5BS</t>
+        </is>
+      </c>
+      <c r="C45" s="26" t="n">
+        <v>110000</v>
+      </c>
+      <c r="D45" s="26">
+        <f>IFERROR(C45*1.2,"")</f>
+        <v>132000.0</v>
+      </c>
+      <c r="E45" s="25" t="n"/>
+      <c r="F45" s="27">
+        <f>IFERROR(D45/E45,"")</f>
+        <v/>
+      </c>
+      <c r="G45" s="25" t="n"/>
+      <c r="H45" s="25" t="n"/>
+      <c r="I45" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="28" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>9 Victoria Road, Margate, Kent, CT9 1LN</t>
+        </is>
+      </c>
+      <c r="C46" s="29" t="n">
+        <v>90000</v>
+      </c>
+      <c r="D46" s="29">
+        <f>IFERROR(C46*1.2,"")</f>
+        <v>108000.0</v>
+      </c>
+      <c r="E46" s="29" t="n">
+        <v>238000</v>
+      </c>
+      <c r="F46" s="30">
+        <f>IFERROR(D46/E46,"")</f>
+        <v>0.4537815126</v>
+      </c>
+      <c r="G46" s="28" t="inlineStr">
+        <is>
+          <t>No offers</t>
+        </is>
+      </c>
+      <c r="H46" s="28" t="inlineStr">
+        <is>
+          <t>Outside region</t>
+        </is>
+      </c>
+      <c r="I46" s="28" t="inlineStr">
+        <is>
+          <t>Yes - Sept lot 42</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="25" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t>2-4 Market Street, Hyde, Cheshire, SK14 1AY</t>
+        </is>
+      </c>
+      <c r="C47" s="26" t="n">
+        <v>90000</v>
+      </c>
+      <c r="D47" s="26">
+        <f>IFERROR(C47*1.2,"")</f>
+        <v>108000.0</v>
+      </c>
+      <c r="E47" s="25" t="n"/>
+      <c r="F47" s="27">
+        <f>IFERROR(D47/E47,"")</f>
+        <v/>
+      </c>
+      <c r="G47" s="25" t="n"/>
+      <c r="H47" s="25" t="n"/>
+      <c r="I47" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="25" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>42 Crumpsall Lane, Manchester, Lancashire, M8 5FB</t>
+        </is>
+      </c>
+      <c r="C48" s="26" t="n">
+        <v>320000</v>
+      </c>
+      <c r="D48" s="26">
+        <f>IFERROR(C48*1.2,"")</f>
+        <v>384000.0</v>
+      </c>
+      <c r="E48" s="25" t="n"/>
+      <c r="F48" s="27">
+        <f>IFERROR(D48/E48,"")</f>
+        <v/>
+      </c>
+      <c r="G48" s="25" t="n"/>
+      <c r="H48" s="25" t="n"/>
+      <c r="I48" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="28" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Flat 4, 280 Wimborne Road, Bournemouth, Dorset, BH3 7AT</t>
+        </is>
+      </c>
+      <c r="C49" s="29" t="n">
+        <v>45000</v>
+      </c>
+      <c r="D49" s="29">
+        <f>IFERROR(C49*1.2,"")</f>
+        <v>54000.0</v>
+      </c>
+      <c r="E49" s="28" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F49" s="30">
+        <f>IFERROR(D49/E49,"")</f>
+        <v/>
+      </c>
+      <c r="G49" s="28" t="n"/>
+      <c r="H49" s="28" t="inlineStr">
+        <is>
+          <t>Outside region</t>
+        </is>
+      </c>
+      <c r="I49" s="28" t="inlineStr">
+        <is>
+          <t>Yes - Sept lot 38</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="25" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>69 Fenton Road, Bournemouth, Dorset, BH6 5BU</t>
+        </is>
+      </c>
+      <c r="C50" s="26" t="n">
+        <v>290000</v>
+      </c>
+      <c r="D50" s="26">
+        <f>IFERROR(C50*1.2,"")</f>
+        <v>348000.0</v>
+      </c>
+      <c r="E50" s="25" t="n"/>
+      <c r="F50" s="27">
+        <f>IFERROR(D50/E50,"")</f>
+        <v/>
+      </c>
+      <c r="G50" s="25" t="n"/>
+      <c r="H50" s="25" t="n"/>
+      <c r="I50" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="25" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>709 Wimborne Road, Bournemouth, Dorset, BH9 2AU</t>
+        </is>
+      </c>
+      <c r="C51" s="26" t="n">
+        <v>350000</v>
+      </c>
+      <c r="D51" s="26">
+        <f>IFERROR(C51*1.2,"")</f>
+        <v>420000.0</v>
+      </c>
+      <c r="E51" s="25" t="n"/>
+      <c r="F51" s="27">
+        <f>IFERROR(D51/E51,"")</f>
+        <v/>
+      </c>
+      <c r="G51" s="25" t="n"/>
+      <c r="H51" s="25" t="n"/>
+      <c r="I51" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="25" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>37 Kent Road, Blackpool, Lancashire, FY1 5HH</t>
+        </is>
+      </c>
+      <c r="C52" s="26" t="n">
+        <v>25000</v>
+      </c>
+      <c r="D52" s="26">
+        <f>IFERROR(C52*1.2,"")</f>
+        <v>30000.0</v>
+      </c>
+      <c r="E52" s="25" t="n"/>
+      <c r="F52" s="27">
+        <f>IFERROR(D52/E52,"")</f>
+        <v/>
+      </c>
+      <c r="G52" s="25" t="n"/>
+      <c r="H52" s="25" t="n"/>
+      <c r="I52" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="28" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>Apartment 006 New Bank House, 100 Queen Street, Sheffield, South Yorkshire, S1 2FA</t>
+        </is>
+      </c>
+      <c r="C53" s="29" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D53" s="29">
+        <f>IFERROR(C53*1.2,"")</f>
+        <v>6000.0</v>
+      </c>
+      <c r="E53" s="29" t="n">
+        <v>58000</v>
+      </c>
+      <c r="F53" s="30">
+        <f>IFERROR(D53/E53,"")</f>
+        <v>0.1034482759</v>
+      </c>
+      <c r="G53" s="29" t="n">
+        <v>35000</v>
+      </c>
+      <c r="H53" s="28" t="inlineStr">
+        <is>
+          <t>Outside region</t>
+        </is>
+      </c>
+      <c r="I53" s="28" t="inlineStr">
+        <is>
+          <t>Yes - Sept lot 166</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="25" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="B54" s="12" t="inlineStr">
+        <is>
+          <t>Telephone Kiosk, Old Town Hall Arches High Street, Reigate, Surrey, RH2 9AA</t>
+        </is>
+      </c>
+      <c r="C54" s="26" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D54" s="26">
+        <f>IFERROR(C54*1.2,"")</f>
+        <v>6000.0</v>
+      </c>
+      <c r="E54" s="25" t="n"/>
+      <c r="F54" s="27">
+        <f>IFERROR(D54/E54,"")</f>
+        <v/>
+      </c>
+      <c r="G54" s="25" t="n"/>
+      <c r="H54" s="25" t="n"/>
+      <c r="I54" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="25" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="B55" s="12" t="inlineStr">
+        <is>
+          <t>Apartment 005 St Peters House, Princes Street, Doncaster, South Yorkshire, DN1 3BP</t>
+        </is>
+      </c>
+      <c r="C55" s="26" t="n">
+        <v>32000</v>
+      </c>
+      <c r="D55" s="26">
+        <f>IFERROR(C55*1.2,"")</f>
+        <v>38400.0</v>
+      </c>
+      <c r="E55" s="25" t="n"/>
+      <c r="F55" s="27">
+        <f>IFERROR(D55/E55,"")</f>
+        <v/>
+      </c>
+      <c r="G55" s="25" t="n"/>
+      <c r="H55" s="25" t="n"/>
+      <c r="I55" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="25" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="B56" s="12" t="inlineStr">
+        <is>
+          <t>Apartment 402 St Peters House, Princes Street, Doncaster, South Yorkshire, DN1 3BP</t>
+        </is>
+      </c>
+      <c r="C56" s="26" t="n">
+        <v>32000</v>
+      </c>
+      <c r="D56" s="26">
+        <f>IFERROR(C56*1.2,"")</f>
+        <v>38400.0</v>
+      </c>
+      <c r="E56" s="25" t="n"/>
+      <c r="F56" s="27">
+        <f>IFERROR(D56/E56,"")</f>
+        <v/>
+      </c>
+      <c r="G56" s="25" t="n"/>
+      <c r="H56" s="25" t="n"/>
+      <c r="I56" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="25" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="B57" s="12" t="inlineStr">
+        <is>
+          <t>111 Benefield Road, Oundle, Peterborough, Cambridgeshire, PE8 4EU</t>
+        </is>
+      </c>
+      <c r="C57" s="26" t="n">
+        <v>145000</v>
+      </c>
+      <c r="D57" s="26">
+        <f>IFERROR(C57*1.2,"")</f>
+        <v>174000.0</v>
+      </c>
+      <c r="E57" s="25" t="n"/>
+      <c r="F57" s="27">
+        <f>IFERROR(D57/E57,"")</f>
+        <v/>
+      </c>
+      <c r="G57" s="25" t="n"/>
+      <c r="H57" s="25" t="n"/>
+      <c r="I57" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="25" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="B58" s="12" t="inlineStr">
+        <is>
+          <t>Catswell Cottage &amp; Adderstone Mains Lodge, Belford, Northumberland, NE70 7HS</t>
+        </is>
+      </c>
+      <c r="C58" s="26" t="n">
+        <v>250000</v>
+      </c>
+      <c r="D58" s="26">
+        <f>IFERROR(C58*1.2,"")</f>
+        <v>300000.0</v>
+      </c>
+      <c r="E58" s="25" t="n"/>
+      <c r="F58" s="27">
+        <f>IFERROR(D58/E58,"")</f>
+        <v/>
+      </c>
+      <c r="G58" s="25" t="n"/>
+      <c r="H58" s="25" t="n"/>
+      <c r="I58" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="25" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="B59" s="12" t="inlineStr">
+        <is>
+          <t>Apartment 71 Dorchester Court, 283 London Road, Camberley, Surrey, GU15 3JJ</t>
+        </is>
+      </c>
+      <c r="C59" s="26" t="n">
+        <v>180000</v>
+      </c>
+      <c r="D59" s="26">
+        <f>IFERROR(C59*1.2,"")</f>
+        <v>216000.0</v>
+      </c>
+      <c r="E59" s="25" t="n"/>
+      <c r="F59" s="27">
+        <f>IFERROR(D59/E59,"")</f>
+        <v/>
+      </c>
+      <c r="G59" s="25" t="n"/>
+      <c r="H59" s="25" t="n"/>
+      <c r="I59" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="25" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="B60" s="12" t="inlineStr">
+        <is>
+          <t>Flat 407 The Printworks, Hodgson Street, Sheffield, South Yorkshire, S3 7WQ</t>
+        </is>
+      </c>
+      <c r="C60" s="26" t="n">
+        <v>20000</v>
+      </c>
+      <c r="D60" s="26">
+        <f>IFERROR(C60*1.2,"")</f>
+        <v>24000.0</v>
+      </c>
+      <c r="E60" s="25" t="n"/>
+      <c r="F60" s="27">
+        <f>IFERROR(D60/E60,"")</f>
+        <v/>
+      </c>
+      <c r="G60" s="25" t="n"/>
+      <c r="H60" s="25" t="n"/>
+      <c r="I60" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="25" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="B61" s="12" t="inlineStr">
+        <is>
+          <t>Flat 408 The Printworks, Hodgson Street, Sheffield, South Yorkshire, S3 7WQ</t>
+        </is>
+      </c>
+      <c r="C61" s="26" t="n">
+        <v>20000</v>
+      </c>
+      <c r="D61" s="26">
+        <f>IFERROR(C61*1.2,"")</f>
+        <v>24000.0</v>
+      </c>
+      <c r="E61" s="25" t="n"/>
+      <c r="F61" s="27">
+        <f>IFERROR(D61/E61,"")</f>
+        <v/>
+      </c>
+      <c r="G61" s="25" t="n"/>
+      <c r="H61" s="25" t="n"/>
+      <c r="I61" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="25" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="B62" s="12" t="inlineStr">
+        <is>
+          <t>The Glynne, Cornist Road, Flint, Clwyd, CH6 5HG</t>
+        </is>
+      </c>
+      <c r="C62" s="26" t="n">
+        <v>140000</v>
+      </c>
+      <c r="D62" s="26">
+        <f>IFERROR(C62*1.2,"")</f>
+        <v>168000.0</v>
+      </c>
+      <c r="E62" s="25" t="n"/>
+      <c r="F62" s="27">
+        <f>IFERROR(D62/E62,"")</f>
+        <v/>
+      </c>
+      <c r="G62" s="25" t="n"/>
+      <c r="H62" s="25" t="n"/>
+      <c r="I62" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="25" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="B63" s="12" t="inlineStr">
+        <is>
+          <t>70 Dutton Lane, Eastleigh, Hampshire, SO50 6AB</t>
+        </is>
+      </c>
+      <c r="C63" s="26" t="n">
+        <v>230000</v>
+      </c>
+      <c r="D63" s="26">
+        <f>IFERROR(C63*1.2,"")</f>
+        <v>276000.0</v>
+      </c>
+      <c r="E63" s="25" t="n"/>
+      <c r="F63" s="27">
+        <f>IFERROR(D63/E63,"")</f>
+        <v/>
+      </c>
+      <c r="G63" s="25" t="n"/>
+      <c r="H63" s="25" t="n"/>
+      <c r="I63" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="25" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="B64" s="12" t="inlineStr">
+        <is>
+          <t>53 Desborough Road, Eastleigh, Hampshire, SO50 5NY</t>
+        </is>
+      </c>
+      <c r="C64" s="26" t="n">
+        <v>250000</v>
+      </c>
+      <c r="D64" s="26">
+        <f>IFERROR(C64*1.2,"")</f>
+        <v>300000.0</v>
+      </c>
+      <c r="E64" s="25" t="n"/>
+      <c r="F64" s="27">
+        <f>IFERROR(D64/E64,"")</f>
+        <v/>
+      </c>
+      <c r="G64" s="25" t="n"/>
+      <c r="H64" s="25" t="n"/>
+      <c r="I64" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="25" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="B65" s="12" t="inlineStr">
+        <is>
+          <t>33 Park View, Sturry, Canterbury, Kent, CT2 0NR</t>
+        </is>
+      </c>
+      <c r="C65" s="26" t="n">
+        <v>150000</v>
+      </c>
+      <c r="D65" s="26">
+        <f>IFERROR(C65*1.2,"")</f>
+        <v>180000.0</v>
+      </c>
+      <c r="E65" s="25" t="n"/>
+      <c r="F65" s="27">
+        <f>IFERROR(D65/E65,"")</f>
+        <v/>
+      </c>
+      <c r="G65" s="25" t="n"/>
+      <c r="H65" s="25" t="n"/>
+      <c r="I65" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="25" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="B66" s="12" t="inlineStr">
+        <is>
+          <t>Flat 428, 2 Moorfields, Liverpool, Merseyside, L2 2BT</t>
+        </is>
+      </c>
+      <c r="C66" s="26" t="n">
+        <v>20000</v>
+      </c>
+      <c r="D66" s="26">
+        <f>IFERROR(C66*1.2,"")</f>
+        <v>24000.0</v>
+      </c>
+      <c r="E66" s="25" t="n"/>
+      <c r="F66" s="27">
+        <f>IFERROR(D66/E66,"")</f>
+        <v/>
+      </c>
+      <c r="G66" s="25" t="n"/>
+      <c r="H66" s="25" t="n"/>
+      <c r="I66" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="25" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="B67" s="12" t="inlineStr">
+        <is>
+          <t>Flat 29 Metro Apartments, 101 Goldsworth Road, Woking, Surrey, GU21 6LF</t>
+        </is>
+      </c>
+      <c r="C67" s="26" t="n">
+        <v>120000</v>
+      </c>
+      <c r="D67" s="26">
+        <f>IFERROR(C67*1.2,"")</f>
+        <v>144000.0</v>
+      </c>
+      <c r="E67" s="25" t="n"/>
+      <c r="F67" s="27">
+        <f>IFERROR(D67/E67,"")</f>
+        <v/>
+      </c>
+      <c r="G67" s="25" t="n"/>
+      <c r="H67" s="25" t="n"/>
+      <c r="I67" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="25" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="B68" s="12" t="inlineStr">
+        <is>
+          <t>Highfields Residential Care Home, Culver Street, Newent, Gloucestershire, GL18 1JA</t>
+        </is>
+      </c>
+      <c r="C68" s="26" t="n">
+        <v>550000</v>
+      </c>
+      <c r="D68" s="26">
+        <f>IFERROR(C68*1.2,"")</f>
+        <v>660000.0</v>
+      </c>
+      <c r="E68" s="25" t="n"/>
+      <c r="F68" s="27">
+        <f>IFERROR(D68/E68,"")</f>
+        <v/>
+      </c>
+      <c r="G68" s="25" t="n"/>
+      <c r="H68" s="25" t="n"/>
+      <c r="I68" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="28" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>Parking Space at 99 Mile End Road, Tower Hamlets, London, E1 4UH</t>
+        </is>
+      </c>
+      <c r="C69" s="29" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D69" s="29">
+        <f>IFERROR(C69*1.2,"")</f>
+        <v>6000.0</v>
+      </c>
+      <c r="E69" s="28" t="inlineStr">
+        <is>
+          <t>N/A - parking</t>
+        </is>
+      </c>
+      <c r="F69" s="30">
+        <f>IFERROR(D69/E69,"")</f>
+        <v/>
+      </c>
+      <c r="G69" s="28" t="n"/>
+      <c r="H69" s="28" t="inlineStr">
+        <is>
+          <t>Outside region</t>
+        </is>
+      </c>
+      <c r="I69" s="28" t="inlineStr">
+        <is>
+          <t>Yes - Sept lot 175</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="25" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B70" s="12" t="inlineStr">
+        <is>
+          <t>Flat 17A Bramley Grange, Horsham Road, Bramley, Guildford, Surrey, GU5 0ES</t>
+        </is>
+      </c>
+      <c r="C70" s="26" t="n">
+        <v>100000</v>
+      </c>
+      <c r="D70" s="26">
+        <f>IFERROR(C70*1.2,"")</f>
+        <v>120000.0</v>
+      </c>
+      <c r="E70" s="25" t="n"/>
+      <c r="F70" s="27">
+        <f>IFERROR(D70/E70,"")</f>
+        <v/>
+      </c>
+      <c r="G70" s="25" t="n"/>
+      <c r="H70" s="25" t="n"/>
+      <c r="I70" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="28" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>Sandly Court, 39 Queens Road, Southport, Merseyside, PR9 9EX</t>
+        </is>
+      </c>
+      <c r="C71" s="29" t="n">
+        <v>320000</v>
+      </c>
+      <c r="D71" s="29">
+        <f>IFERROR(C71*1.2,"")</f>
+        <v>384000.0</v>
+      </c>
+      <c r="E71" s="28" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F71" s="30">
+        <f>IFERROR(D71/E71,"")</f>
+        <v/>
+      </c>
+      <c r="G71" s="28" t="n"/>
+      <c r="H71" s="28" t="inlineStr">
+        <is>
+          <t>CLOSED + NW paused</t>
+        </is>
+      </c>
+      <c r="I71" s="28" t="inlineStr">
+        <is>
+          <t>Yes - Sept lot 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="25" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
+      <c r="B72" s="12" t="inlineStr">
+        <is>
+          <t>7 Mansfield Road, Doncaster, South Yorkshire, DN4 0LG</t>
+        </is>
+      </c>
+      <c r="C72" s="26" t="n">
+        <v>70000</v>
+      </c>
+      <c r="D72" s="26">
+        <f>IFERROR(C72*1.2,"")</f>
+        <v>84000.0</v>
+      </c>
+      <c r="E72" s="25" t="n"/>
+      <c r="F72" s="27">
+        <f>IFERROR(D72/E72,"")</f>
+        <v/>
+      </c>
+      <c r="G72" s="25" t="n"/>
+      <c r="H72" s="25" t="n"/>
+      <c r="I72" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="31" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="B73" s="8" t="inlineStr">
+        <is>
+          <t>48 High East Street, Dorchester, Dorset, DT1 1HU</t>
+        </is>
+      </c>
+      <c r="C73" s="31" t="n"/>
+      <c r="D73" s="32">
+        <f>IFERROR(C73*1.2,"")</f>
+        <v/>
+      </c>
+      <c r="E73" s="31" t="n"/>
+      <c r="F73" s="33">
+        <f>IFERROR(D73/E73,"")</f>
+        <v/>
+      </c>
+      <c r="G73" s="31" t="n"/>
+      <c r="H73" s="31" t="n"/>
+      <c r="I73" s="31" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="25" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
+      </c>
+      <c r="B74" s="12" t="inlineStr">
+        <is>
+          <t>66-70 High Street, Mexborough, Doncaster, S64 9AU</t>
+        </is>
+      </c>
+      <c r="C74" s="26" t="n">
+        <v>145000</v>
+      </c>
+      <c r="D74" s="26">
+        <f>IFERROR(C74*1.2,"")</f>
+        <v>174000.0</v>
+      </c>
+      <c r="E74" s="25" t="n"/>
+      <c r="F74" s="27">
+        <f>IFERROR(D74/E74,"")</f>
+        <v/>
+      </c>
+      <c r="G74" s="25" t="n"/>
+      <c r="H74" s="25" t="n"/>
+      <c r="I74" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="28" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>Flat 105, 2 Moorfields, Liverpool, Merseyside, L2 2BS</t>
+        </is>
+      </c>
+      <c r="C75" s="29" t="n">
+        <v>20000</v>
+      </c>
+      <c r="D75" s="29">
+        <f>IFERROR(C75*1.2,"")</f>
+        <v>24000.0</v>
+      </c>
+      <c r="E75" s="29" t="n">
+        <v>90000</v>
+      </c>
+      <c r="F75" s="30">
+        <f>IFERROR(D75/E75,"")</f>
+        <v>0.2666666667</v>
+      </c>
+      <c r="G75" s="29" t="n">
+        <v>40000</v>
+      </c>
+      <c r="H75" s="28" t="inlineStr">
+        <is>
+          <t>CLOSED + NW paused</t>
+        </is>
+      </c>
+      <c r="I75" s="28" t="inlineStr">
+        <is>
+          <t>Yes - Sept lot 112</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="28" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>Parking Space 31 Lollard Street, Lambeth, London, SE11 6PX</t>
+        </is>
+      </c>
+      <c r="C76" s="29" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D76" s="29">
+        <f>IFERROR(C76*1.2,"")</f>
+        <v>6000.0</v>
+      </c>
+      <c r="E76" s="28" t="inlineStr">
+        <is>
+          <t>N/A - parking</t>
+        </is>
+      </c>
+      <c r="F76" s="30">
+        <f>IFERROR(D76/E76,"")</f>
+        <v/>
+      </c>
+      <c r="G76" s="28" t="n"/>
+      <c r="H76" s="28" t="inlineStr">
+        <is>
+          <t>Outside region</t>
+        </is>
+      </c>
+      <c r="I76" s="28" t="inlineStr">
+        <is>
+          <t>Yes - Sept lot 160</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="25" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="B77" s="12" t="inlineStr">
+        <is>
+          <t>Garage 5, 28 Braidley Road, Bournemouth, Dorset, BH2 6JX</t>
+        </is>
+      </c>
+      <c r="C77" s="26" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D77" s="26">
+        <f>IFERROR(C77*1.2,"")</f>
+        <v>6000.0</v>
+      </c>
+      <c r="E77" s="25" t="n"/>
+      <c r="F77" s="27">
+        <f>IFERROR(D77/E77,"")</f>
+        <v/>
+      </c>
+      <c r="G77" s="25" t="n"/>
+      <c r="H77" s="25" t="n"/>
+      <c r="I77" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="31" t="inlineStr">
+        <is>
+          <t>77</t>
+        </is>
+      </c>
+      <c r="B78" s="8" t="inlineStr">
+        <is>
+          <t>Garage at 1 The Chestnuts, Gwydor Road, Beckenham, Kent, BR3 4DU</t>
+        </is>
+      </c>
+      <c r="C78" s="32" t="n">
+        <v>8000</v>
+      </c>
+      <c r="D78" s="32">
+        <f>IFERROR(C78*1.2,"")</f>
+        <v>9600.0</v>
+      </c>
+      <c r="E78" s="31" t="inlineStr">
+        <is>
+          <t>N/A - garage</t>
+        </is>
+      </c>
+      <c r="F78" s="33">
+        <f>IFERROR(D78/E78,"")</f>
+        <v/>
+      </c>
+      <c r="G78" s="31" t="n"/>
+      <c r="H78" s="31" t="inlineStr">
+        <is>
+          <t>Outside region</t>
+        </is>
+      </c>
+      <c r="I78" s="31" t="inlineStr">
+        <is>
+          <t>Yes - Sept lot 127</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="25" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="B79" s="12" t="inlineStr">
+        <is>
+          <t>Garage at Chestnut Court, 14 Lancaster Road, South Norwood, London, SE25 4AH</t>
+        </is>
+      </c>
+      <c r="C79" s="26" t="n">
+        <v>10000</v>
+      </c>
+      <c r="D79" s="26">
+        <f>IFERROR(C79*1.2,"")</f>
+        <v>12000.0</v>
+      </c>
+      <c r="E79" s="25" t="n"/>
+      <c r="F79" s="27">
+        <f>IFERROR(D79/E79,"")</f>
+        <v/>
+      </c>
+      <c r="G79" s="25" t="n"/>
+      <c r="H79" s="25" t="n"/>
+      <c r="I79" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="25" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="B80" s="12" t="inlineStr">
+        <is>
+          <t>Garage 11, 62 Oxenden Road, Tongham, Farnham, Surrey, GU10 1AJ</t>
+        </is>
+      </c>
+      <c r="C80" s="26" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D80" s="26">
+        <f>IFERROR(C80*1.2,"")</f>
+        <v>3600.0</v>
+      </c>
+      <c r="E80" s="25" t="n"/>
+      <c r="F80" s="27">
+        <f>IFERROR(D80/E80,"")</f>
+        <v/>
+      </c>
+      <c r="G80" s="25" t="n"/>
+      <c r="H80" s="25" t="n"/>
+      <c r="I80" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="25" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="B81" s="12" t="inlineStr">
+        <is>
+          <t>Garage at 32 Brussels Way, Luton, Bedfordshire, LU3 3TQ</t>
+        </is>
+      </c>
+      <c r="C81" s="26" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D81" s="26">
+        <f>IFERROR(C81*1.2,"")</f>
+        <v>6000.0</v>
+      </c>
+      <c r="E81" s="25" t="n"/>
+      <c r="F81" s="27">
+        <f>IFERROR(D81/E81,"")</f>
+        <v/>
+      </c>
+      <c r="G81" s="25" t="n"/>
+      <c r="H81" s="25" t="n"/>
+      <c r="I81" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="25" t="inlineStr">
+        <is>
+          <t>81</t>
+        </is>
+      </c>
+      <c r="B82" s="12" t="inlineStr">
+        <is>
+          <t>Garages and Land at Regent Street, Stowmarket, Suffolk, IP14 1RJ</t>
+        </is>
+      </c>
+      <c r="C82" s="26" t="n">
+        <v>40000</v>
+      </c>
+      <c r="D82" s="26">
+        <f>IFERROR(C82*1.2,"")</f>
+        <v>48000.0</v>
+      </c>
+      <c r="E82" s="25" t="n"/>
+      <c r="F82" s="27">
+        <f>IFERROR(D82/E82,"")</f>
+        <v/>
+      </c>
+      <c r="G82" s="25" t="n"/>
+      <c r="H82" s="25" t="n"/>
+      <c r="I82" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="25" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
+      </c>
+      <c r="B83" s="12" t="inlineStr">
+        <is>
+          <t>Garage 31 at Blackabrook Avenue, Princetown, Yelverton, Devon, PL20 6RH</t>
+        </is>
+      </c>
+      <c r="C83" s="26" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D83" s="26">
+        <f>IFERROR(C83*1.2,"")</f>
+        <v>1200.0</v>
+      </c>
+      <c r="E83" s="25" t="n"/>
+      <c r="F83" s="27">
+        <f>IFERROR(D83/E83,"")</f>
+        <v/>
+      </c>
+      <c r="G83" s="25" t="n"/>
+      <c r="H83" s="25" t="n"/>
+      <c r="I83" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="25" t="inlineStr">
+        <is>
+          <t>83</t>
+        </is>
+      </c>
+      <c r="B84" s="12" t="inlineStr">
+        <is>
+          <t>Land at Law Hall Cottages, Bendish, Hitchin, Hertfordshire, SG4 8JG</t>
+        </is>
+      </c>
+      <c r="C84" s="26" t="n">
+        <v>65000</v>
+      </c>
+      <c r="D84" s="26">
+        <f>IFERROR(C84*1.2,"")</f>
+        <v>78000.0</v>
+      </c>
+      <c r="E84" s="25" t="n"/>
+      <c r="F84" s="27">
+        <f>IFERROR(D84/E84,"")</f>
+        <v/>
+      </c>
+      <c r="G84" s="25" t="n"/>
+      <c r="H84" s="25" t="n"/>
+      <c r="I84" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="25" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="B85" s="12" t="inlineStr">
+        <is>
+          <t>Land Adjacent to 14 Littledale Green Street Green Road, Lane End, Dartford, Kent, DA2 7HU</t>
+        </is>
+      </c>
+      <c r="C85" s="26" t="n">
+        <v>20000</v>
+      </c>
+      <c r="D85" s="26">
+        <f>IFERROR(C85*1.2,"")</f>
+        <v>24000.0</v>
+      </c>
+      <c r="E85" s="25" t="n"/>
+      <c r="F85" s="27">
+        <f>IFERROR(D85/E85,"")</f>
+        <v/>
+      </c>
+      <c r="G85" s="25" t="n"/>
+      <c r="H85" s="25" t="n"/>
+      <c r="I85" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="25" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="B86" s="12" t="inlineStr">
+        <is>
+          <t>Former School, Lea Road, Gainsborough, Lincolnshire, DN21 1AF</t>
+        </is>
+      </c>
+      <c r="C86" s="26" t="n">
+        <v>100000</v>
+      </c>
+      <c r="D86" s="26">
+        <f>IFERROR(C86*1.2,"")</f>
+        <v>120000.0</v>
+      </c>
+      <c r="E86" s="25" t="n"/>
+      <c r="F86" s="27">
+        <f>IFERROR(D86/E86,"")</f>
+        <v/>
+      </c>
+      <c r="G86" s="25" t="n"/>
+      <c r="H86" s="25" t="n"/>
+      <c r="I86" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="25" t="inlineStr">
+        <is>
+          <t>86</t>
+        </is>
+      </c>
+      <c r="B87" s="12" t="inlineStr">
+        <is>
+          <t>Land Adjacent to Silverbank, Chatham, Kent, ME5 0LQ</t>
+        </is>
+      </c>
+      <c r="C87" s="26" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D87" s="26">
+        <f>IFERROR(C87*1.2,"")</f>
+        <v>2400.0</v>
+      </c>
+      <c r="E87" s="25" t="n"/>
+      <c r="F87" s="27">
+        <f>IFERROR(D87/E87,"")</f>
+        <v/>
+      </c>
+      <c r="G87" s="25" t="n"/>
+      <c r="H87" s="25" t="n"/>
+      <c r="I87" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="31" t="inlineStr">
+        <is>
+          <t>87</t>
+        </is>
+      </c>
+      <c r="B88" s="8" t="inlineStr">
+        <is>
+          <t>Land to the Rear of 103 Church Street, Broadstairs, Kent, CT10 2TX</t>
+        </is>
+      </c>
+      <c r="C88" s="31" t="n"/>
+      <c r="D88" s="32">
+        <f>IFERROR(C88*1.2,"")</f>
+        <v/>
+      </c>
+      <c r="E88" s="31" t="inlineStr">
+        <is>
+          <t>N/A - land</t>
+        </is>
+      </c>
+      <c r="F88" s="33">
+        <f>IFERROR(D88/E88,"")</f>
+        <v/>
+      </c>
+      <c r="G88" s="31" t="n"/>
+      <c r="H88" s="31" t="inlineStr">
+        <is>
+          <t>Outside region</t>
+        </is>
+      </c>
+      <c r="I88" s="31" t="inlineStr">
+        <is>
+          <t>Yes - Sept lot 182</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="25" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="B89" s="12" t="inlineStr">
+        <is>
+          <t>Land Adjacent to 50 Camelot Close, Thamesmead, London, SE28 0ET</t>
+        </is>
+      </c>
+      <c r="C89" s="26" t="n">
+        <v>85000</v>
+      </c>
+      <c r="D89" s="26">
+        <f>IFERROR(C89*1.2,"")</f>
+        <v>102000.0</v>
+      </c>
+      <c r="E89" s="25" t="n"/>
+      <c r="F89" s="27">
+        <f>IFERROR(D89/E89,"")</f>
+        <v/>
+      </c>
+      <c r="G89" s="25" t="n"/>
+      <c r="H89" s="25" t="n"/>
+      <c r="I89" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="25" t="inlineStr">
+        <is>
+          <t>89</t>
+        </is>
+      </c>
+      <c r="B90" s="12" t="inlineStr">
+        <is>
+          <t>Land Adjacent to 27 Highgate, Nelson, Lancashire, BB9 0DU</t>
+        </is>
+      </c>
+      <c r="C90" s="26" t="n">
+        <v>185000</v>
+      </c>
+      <c r="D90" s="26">
+        <f>IFERROR(C90*1.2,"")</f>
+        <v>222000.0</v>
+      </c>
+      <c r="E90" s="25" t="n"/>
+      <c r="F90" s="27">
+        <f>IFERROR(D90/E90,"")</f>
+        <v/>
+      </c>
+      <c r="G90" s="25" t="n"/>
+      <c r="H90" s="25" t="n"/>
+      <c r="I90" s="25" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="31" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="B91" s="8" t="inlineStr">
+        <is>
+          <t>81B High Street, Whitton, Twickenham, Middlesex, TW2 7LD</t>
+        </is>
+      </c>
+      <c r="C91" s="31" t="n"/>
+      <c r="D91" s="32">
+        <f>IFERROR(C91*1.2,"")</f>
+        <v/>
+      </c>
+      <c r="E91" s="31" t="n"/>
+      <c r="F91" s="33">
+        <f>IFERROR(D91/E91,"")</f>
+        <v/>
+      </c>
+      <c r="G91" s="31" t="n"/>
+      <c r="H91" s="31" t="n"/>
+      <c r="I91" s="31" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="31" t="inlineStr">
+        <is>
+          <t>91</t>
+        </is>
+      </c>
+      <c r="B92" s="8" t="inlineStr">
+        <is>
+          <t>Hambridge Mill, Hambridge, Langport, Somerset, TA10 0BP</t>
+        </is>
+      </c>
+      <c r="C92" s="31" t="n"/>
+      <c r="D92" s="32">
+        <f>IFERROR(C92*1.2,"")</f>
+        <v/>
+      </c>
+      <c r="E92" s="31" t="n"/>
+      <c r="F92" s="33">
+        <f>IFERROR(D92/E92,"")</f>
+        <v/>
+      </c>
+      <c r="G92" s="31" t="n"/>
+      <c r="H92" s="31" t="n"/>
+      <c r="I92" s="31" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="31" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="B93" s="8" t="inlineStr">
+        <is>
+          <t>34 Whaddon Road, Cheltenham, Gloucestershire, GL52 5NA</t>
+        </is>
+      </c>
+      <c r="C93" s="31" t="n"/>
+      <c r="D93" s="32">
+        <f>IFERROR(C93*1.2,"")</f>
+        <v/>
+      </c>
+      <c r="E93" s="31" t="n"/>
+      <c r="F93" s="33">
+        <f>IFERROR(D93/E93,"")</f>
+        <v/>
+      </c>
+      <c r="G93" s="31" t="n"/>
+      <c r="H93" s="31" t="n"/>
+      <c r="I93" s="31" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="31" t="inlineStr">
+        <is>
+          <t>93</t>
+        </is>
+      </c>
+      <c r="B94" s="8" t="inlineStr">
+        <is>
+          <t>44 Newton Nottage Road, Porthcawl, Mid Glamorgan, CF36 5RP</t>
+        </is>
+      </c>
+      <c r="C94" s="31" t="n"/>
+      <c r="D94" s="32">
+        <f>IFERROR(C94*1.2,"")</f>
+        <v/>
+      </c>
+      <c r="E94" s="31" t="n"/>
+      <c r="F94" s="33">
+        <f>IFERROR(D94/E94,"")</f>
+        <v/>
+      </c>
+      <c r="G94" s="31" t="n"/>
+      <c r="H94" s="31" t="n"/>
+      <c r="I94" s="31" t="inlineStr">
+        <is>
+          <t>New - not in our September list</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I94"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3331,7 +6400,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9218,7 +12287,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>